<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/09/2026 06:21:10
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,22 +513,22 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -683,12 +683,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -902,17 +902,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1877</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1817</t>
+          <t>1815</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1953</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1953</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1953</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2054,17 +2054,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2246,17 +2246,17 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2374,17 +2374,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2438,17 +2438,17 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1850</t>
+          <t>1848</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2758,17 +2758,17 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>280826111844285</t>
+          <t>280826060740757</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2822,17 +2822,17 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>280826060740757</t>
+          <t>280826111844285</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2945,22 +2945,22 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CAL-026-006-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-006-001</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3824,7 +3824,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1921</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1921</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1877</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1848</t>
+          <t>1846</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1926</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1986</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1864</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1864</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1864</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1863</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13766,7 +13766,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -14086,7 +14086,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -14534,7 +14534,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -14598,7 +14598,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -14726,7 +14726,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -14790,7 +14790,7 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
@@ -14854,7 +14854,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -14918,7 +14918,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -15046,7 +15046,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -15302,7 +15302,7 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -15430,7 +15430,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -15622,7 +15622,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -15686,7 +15686,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15750,7 +15750,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -15814,7 +15814,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -15942,7 +15942,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -16006,7 +16006,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -16070,7 +16070,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -16198,7 +16198,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -16262,7 +16262,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -16390,7 +16390,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -16582,7 +16582,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -16646,7 +16646,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -16774,7 +16774,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -16966,7 +16966,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -17030,7 +17030,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -17094,7 +17094,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -17158,7 +17158,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -17222,7 +17222,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -17350,7 +17350,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -17414,7 +17414,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>1926</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -17478,7 +17478,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -17542,7 +17542,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -17606,7 +17606,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -17734,7 +17734,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -17798,7 +17798,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>1864</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -17862,7 +17862,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -17926,7 +17926,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -18054,7 +18054,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -18118,7 +18118,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -18182,7 +18182,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -18246,7 +18246,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>1864</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>1954</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -18374,7 +18374,7 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>1796</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>1864</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -18502,7 +18502,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>1954</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>1864</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -18630,7 +18630,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>1954</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -18694,7 +18694,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -18758,7 +18758,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -18822,7 +18822,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -18886,7 +18886,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>1914</t>
+          <t>1912</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/09/2026 07:42:43
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N280"/>
+  <dimension ref="A1:N277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6027,12 +6027,12 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6091,12 +6091,12 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6699,12 +6699,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6763,12 +6763,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C100" t="inlineStr"/>
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -9323,12 +9323,12 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
@@ -9345,27 +9345,27 @@
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -9375,7 +9375,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -9387,12 +9387,12 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
@@ -9409,27 +9409,27 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9473,27 +9473,27 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9601,27 +9601,27 @@
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9665,27 +9665,27 @@
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9899,12 +9899,12 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C149" t="inlineStr"/>
@@ -9921,27 +9921,27 @@
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -9985,27 +9985,27 @@
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10177,27 +10177,27 @@
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -10241,27 +10241,27 @@
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10347,12 +10347,12 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
@@ -10369,27 +10369,27 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>110826062045244</t>
+          <t>110826072521981</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>110826072521949</t>
+          <t>110826072522043</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>110826062045384</t>
+          <t>110826062045291</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>110826072521996</t>
+          <t>110826062045244</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>110826072521981</t>
+          <t>110826062045259</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>110826062045259</t>
+          <t>110826072521934</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11531,12 +11531,12 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>110826072522028</t>
+          <t>110826072521965</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>110826062045291</t>
+          <t>110826072521949</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>110826072521965</t>
+          <t>110826062045384</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>110826072521934</t>
+          <t>110826072522028</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11856,7 +11856,7 @@
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>110826072522043</t>
+          <t>110826072521996</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -12171,12 +12171,12 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12299,12 +12299,12 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12464,7 +12464,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12656,7 +12656,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
@@ -12673,22 +12673,22 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12784,7 +12784,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
@@ -12801,22 +12801,22 @@
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12848,7 +12848,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
@@ -12865,22 +12865,22 @@
       <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -13003,12 +13003,12 @@
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
@@ -13067,12 +13067,12 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13087,7 +13087,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
@@ -13121,22 +13121,22 @@
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -13185,22 +13185,22 @@
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>110826062046369</t>
+          <t>110826062045525</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>110826062045978</t>
+          <t>110826062045931</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>110826062045697</t>
+          <t>110826062046119</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>110826062045916</t>
+          <t>110826062046025</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>110826062045869</t>
+          <t>110826062045791</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>110826062045509</t>
+          <t>110826062045431</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>110826062045400</t>
+          <t>110826062046041</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>110826062046291</t>
+          <t>110826062045369</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>110826062046103</t>
+          <t>110826062045541</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>110826062045416</t>
+          <t>110826062045494</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>110826062045759</t>
+          <t>110826062045338</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>110826062045838</t>
+          <t>110826062045775</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>110826062045463</t>
+          <t>110826062046400</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>110826062046400</t>
+          <t>110826062046322</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>110826062045775</t>
+          <t>110826062045463</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>110826062045338</t>
+          <t>110826062045838</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>110826062045369</t>
+          <t>110826062045759</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>110826062046041</t>
+          <t>110826062045416</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>110826062045431</t>
+          <t>110826062045556</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>110826062045791</t>
+          <t>110826062046103</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>110826062046025</t>
+          <t>110826062045963</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>110826062046119</t>
+          <t>110826062046291</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>110826062045931</t>
+          <t>110826062045400</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>110826062045525</t>
+          <t>110826062045509</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>110826062045822</t>
+          <t>110826062046369</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>110826062046275</t>
+          <t>110826062045353</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>110826062045572</t>
+          <t>110826062045978</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14987,12 +14987,12 @@
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>110826062046338</t>
+          <t>110826062045306</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15007,7 +15007,7 @@
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>110826062045541</t>
+          <t>110826062046072</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>110826062045478</t>
+          <t>110826062045994</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15179,12 +15179,12 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>110826062045681</t>
+          <t>110826062045853</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15199,7 +15199,7 @@
       </c>
       <c r="M231" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N231" t="inlineStr">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>110826062045494</t>
+          <t>110826062046306</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>110826062046088</t>
+          <t>110826062045884</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>110826062046353</t>
+          <t>110826062045806</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>110826062045963</t>
+          <t>110826062045322</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>110826062045322</t>
+          <t>110826062045728</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15627,12 +15627,12 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>110826062045806</t>
+          <t>110826062045447</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15647,7 +15647,7 @@
       </c>
       <c r="M238" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N238" t="inlineStr">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>110826062046306</t>
+          <t>110826062046353</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>110826062045994</t>
+          <t>110826062046009</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>110826062046072</t>
+          <t>110826062046088</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15883,12 +15883,12 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>110826062045306</t>
+          <t>110826062045681</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15903,7 +15903,7 @@
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>110826062046322</t>
+          <t>110826062045478</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -16016,7 +16016,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>110826062045556</t>
+          <t>110826062046338</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16080,7 +16080,7 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>110826062045884</t>
+          <t>110826062045572</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16144,7 +16144,7 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>110826062045853</t>
+          <t>110826062045947</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16203,12 +16203,12 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>110826062045447</t>
+          <t>110826062045822</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -16223,7 +16223,7 @@
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N247" t="inlineStr">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>110826062046259</t>
+          <t>110826062045869</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>110826062046009</t>
+          <t>110826062045916</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>110826062046244</t>
+          <t>110826062045697</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -16432,39 +16432,39 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C251" t="inlineStr"/>
       <c r="D251" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101P-1      </t>
+          <t xml:space="preserve">INO102-1       </t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
         </is>
       </c>
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>110826062045728</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16479,7 +16479,7 @@
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N251" t="inlineStr">
@@ -16496,39 +16496,39 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C252" t="inlineStr"/>
       <c r="D252" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101P-1      </t>
+          <t xml:space="preserve">INO102-1       </t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
         </is>
       </c>
       <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>110826062045947</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -16543,7 +16543,7 @@
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N252" t="inlineStr">
@@ -16560,39 +16560,39 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C253" t="inlineStr"/>
       <c r="D253" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101P-1      </t>
+          <t xml:space="preserve">INO102-1       </t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
         </is>
       </c>
       <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
         <is>
-          <t>110826062045353</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K253" t="inlineStr">
@@ -16607,7 +16607,7 @@
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N253" t="inlineStr">
@@ -16641,22 +16641,22 @@
       <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -16671,7 +16671,7 @@
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N254" t="inlineStr">
@@ -16715,12 +16715,12 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
@@ -16758,33 +16758,33 @@
       <c r="C256" t="inlineStr"/>
       <c r="D256" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-1       </t>
+          <t xml:space="preserve">INO102-2       </t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16799,7 +16799,7 @@
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N256" t="inlineStr">
@@ -16816,39 +16816,39 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C257" t="inlineStr"/>
       <c r="D257" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-1       </t>
+          <t xml:space="preserve">INO102-2       </t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16863,7 +16863,7 @@
       </c>
       <c r="M257" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N257" t="inlineStr">
@@ -16880,39 +16880,39 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C258" t="inlineStr"/>
       <c r="D258" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-1       </t>
+          <t xml:space="preserve">INO103-2       </t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
         </is>
       </c>
       <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>MMQT4</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16927,7 +16927,7 @@
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N258" t="inlineStr">
@@ -16944,39 +16944,39 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C259" t="inlineStr"/>
       <c r="D259" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-2       </t>
+          <t xml:space="preserve">INO104-1       </t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
         </is>
       </c>
       <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -16991,7 +16991,7 @@
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N259" t="inlineStr">
@@ -17014,33 +17014,33 @@
       <c r="C260" t="inlineStr"/>
       <c r="D260" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-2       </t>
+          <t xml:space="preserve">INO104-1       </t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
         </is>
       </c>
       <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -17055,7 +17055,7 @@
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N260" t="inlineStr">
@@ -17072,39 +17072,39 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C261" t="inlineStr"/>
       <c r="D261" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO103-2       </t>
+          <t xml:space="preserve">INO104-1       </t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
         </is>
       </c>
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>MMQT4</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17119,7 +17119,7 @@
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N261" t="inlineStr">
@@ -17142,12 +17142,12 @@
       <c r="C262" t="inlineStr"/>
       <c r="D262" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-1       </t>
+          <t xml:space="preserve">INO104-2       </t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
         </is>
       </c>
       <c r="F262" t="inlineStr"/>
@@ -17163,12 +17163,12 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -17183,7 +17183,7 @@
       </c>
       <c r="M262" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N262" t="inlineStr">
@@ -17206,33 +17206,33 @@
       <c r="C263" t="inlineStr"/>
       <c r="D263" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-1       </t>
+          <t xml:space="preserve">INO104-2       </t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
         </is>
       </c>
       <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056680</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -17247,7 +17247,7 @@
       </c>
       <c r="M263" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="N263" t="inlineStr">
@@ -17270,12 +17270,12 @@
       <c r="C264" t="inlineStr"/>
       <c r="D264" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-1       </t>
+          <t xml:space="preserve">INO104N-1      </t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
+          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
         </is>
       </c>
       <c r="F264" t="inlineStr"/>
@@ -17291,12 +17291,12 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -17311,7 +17311,7 @@
       </c>
       <c r="M264" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N264" t="inlineStr">
@@ -17334,12 +17334,12 @@
       <c r="C265" t="inlineStr"/>
       <c r="D265" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-2       </t>
+          <t xml:space="preserve">INO104N-1      </t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
+          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
         </is>
       </c>
       <c r="F265" t="inlineStr"/>
@@ -17355,12 +17355,12 @@
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -17375,7 +17375,7 @@
       </c>
       <c r="M265" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N265" t="inlineStr">
@@ -17392,39 +17392,39 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C266" t="inlineStr"/>
       <c r="D266" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-2       </t>
+          <t xml:space="preserve">INO104N-1      </t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
+          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
         </is>
       </c>
       <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>180226073056680</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -17439,7 +17439,7 @@
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N266" t="inlineStr">
@@ -17456,7 +17456,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C267" t="inlineStr"/>
@@ -17473,22 +17473,22 @@
       <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J267" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -17503,7 +17503,7 @@
       </c>
       <c r="M267" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N267" t="inlineStr">
@@ -17520,7 +17520,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C268" t="inlineStr"/>
@@ -17537,22 +17537,22 @@
       <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -17567,7 +17567,7 @@
       </c>
       <c r="M268" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N268" t="inlineStr">
@@ -17584,7 +17584,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C269" t="inlineStr"/>
@@ -17601,22 +17601,22 @@
       <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K269" t="inlineStr">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="M269" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N269" t="inlineStr">
@@ -17648,39 +17648,39 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C270" t="inlineStr"/>
       <c r="D270" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -17695,7 +17695,7 @@
       </c>
       <c r="M270" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N270" t="inlineStr">
@@ -17718,33 +17718,33 @@
       <c r="C271" t="inlineStr"/>
       <c r="D271" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -17759,7 +17759,7 @@
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N271" t="inlineStr">
@@ -17776,39 +17776,39 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C272" t="inlineStr"/>
       <c r="D272" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -17823,7 +17823,7 @@
       </c>
       <c r="M272" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N272" t="inlineStr">
@@ -17840,39 +17840,39 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C273" t="inlineStr"/>
       <c r="D273" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U1133G         </t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
         </is>
       </c>
       <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>22/11/2031</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>300</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -17887,7 +17887,7 @@
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>300</t>
         </is>
       </c>
       <c r="N273" t="inlineStr">
@@ -17904,44 +17904,44 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C274" t="inlineStr"/>
       <c r="D274" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U889-01        </t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
         </is>
       </c>
       <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>09/12/2031</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1912</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>180626072347907</t>
         </is>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L274" t="inlineStr">
@@ -17951,7 +17951,7 @@
       </c>
       <c r="M274" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>50</t>
         </is>
       </c>
       <c r="N274" t="inlineStr">
@@ -17968,39 +17968,39 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C275" t="inlineStr"/>
       <c r="D275" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U889-01        </t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
         </is>
       </c>
       <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -18015,7 +18015,7 @@
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N275" t="inlineStr">
@@ -18038,28 +18038,28 @@
       <c r="C276" t="inlineStr"/>
       <c r="D276" t="inlineStr">
         <is>
-          <t xml:space="preserve">U1133G         </t>
+          <t xml:space="preserve">U891           </t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
+          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
         </is>
       </c>
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
-          <t>22/11/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
@@ -18079,7 +18079,7 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N276" t="inlineStr">
@@ -18102,38 +18102,38 @@
       <c r="C277" t="inlineStr"/>
       <c r="D277" t="inlineStr">
         <is>
-          <t xml:space="preserve">U889-01        </t>
+          <t xml:space="preserve">U948-1         </t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
+          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
         </is>
       </c>
       <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
-          <t>09/12/2031</t>
+          <t>31/01/2032</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>1912</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>507</t>
         </is>
       </c>
       <c r="J277" t="inlineStr">
         <is>
-          <t>180626072347907</t>
+          <t>100826061846740</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
@@ -18143,202 +18143,10 @@
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>507</t>
         </is>
       </c>
       <c r="N277" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>CAL-027-008-001</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr"/>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U889-01        </t>
-        </is>
-      </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
-        </is>
-      </c>
-      <c r="F278" t="inlineStr"/>
-      <c r="G278" t="inlineStr">
-        <is>
-          <t>03/11/2031</t>
-        </is>
-      </c>
-      <c r="H278" t="inlineStr">
-        <is>
-          <t>1876</t>
-        </is>
-      </c>
-      <c r="I278" t="inlineStr">
-        <is>
-          <t>77</t>
-        </is>
-      </c>
-      <c r="J278" t="inlineStr">
-        <is>
-          <t>110226132440294</t>
-        </is>
-      </c>
-      <c r="K278" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L278" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M278" t="inlineStr">
-        <is>
-          <t>77</t>
-        </is>
-      </c>
-      <c r="N278" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>CAL-027-008-001</t>
-        </is>
-      </c>
-      <c r="C279" t="inlineStr"/>
-      <c r="D279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U891           </t>
-        </is>
-      </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
-        </is>
-      </c>
-      <c r="F279" t="inlineStr"/>
-      <c r="G279" t="inlineStr">
-        <is>
-          <t>03/11/2031</t>
-        </is>
-      </c>
-      <c r="H279" t="inlineStr">
-        <is>
-          <t>1876</t>
-        </is>
-      </c>
-      <c r="I279" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="J279" t="inlineStr">
-        <is>
-          <t>110226132440294</t>
-        </is>
-      </c>
-      <c r="K279" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L279" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M279" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="N279" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>CAL-001-001-001</t>
-        </is>
-      </c>
-      <c r="C280" t="inlineStr"/>
-      <c r="D280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U948-1         </t>
-        </is>
-      </c>
-      <c r="E280" t="inlineStr">
-        <is>
-          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
-        </is>
-      </c>
-      <c r="F280" t="inlineStr"/>
-      <c r="G280" t="inlineStr">
-        <is>
-          <t>31/01/2032</t>
-        </is>
-      </c>
-      <c r="H280" t="inlineStr">
-        <is>
-          <t>1965</t>
-        </is>
-      </c>
-      <c r="I280" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="J280" t="inlineStr">
-        <is>
-          <t>100826061846740</t>
-        </is>
-      </c>
-      <c r="K280" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L280" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M280" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="N280" t="inlineStr">
         <is>
           <t>NO</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/09/2026 08:37:35
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N264"/>
+  <dimension ref="A1:N261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3585,22 +3585,22 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4481,12 +4481,12 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4737,22 +4737,22 @@
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5185,22 +5185,22 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5313,12 +5313,12 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5377,12 +5377,12 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5441,12 +5441,12 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5569,12 +5569,12 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5633,12 +5633,12 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5697,12 +5697,12 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5761,22 +5761,22 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5835,12 +5835,12 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5953,12 +5953,12 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,12 +6081,12 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6187,12 +6187,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6315,12 +6315,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -6347,12 +6347,12 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -6379,12 +6379,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6443,12 +6443,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6507,12 +6507,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -6539,12 +6539,12 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6559,7 +6559,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -6571,12 +6571,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6699,12 +6699,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6763,12 +6763,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C100" t="inlineStr"/>
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7376,12 +7376,12 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7435,12 +7435,12 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7489,27 +7489,27 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7681,27 +7681,27 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7809,27 +7809,27 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -7888,12 +7888,12 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7937,27 +7937,27 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8065,27 +8065,27 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -8129,27 +8129,27 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8449,27 +8449,27 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8491,12 +8491,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
@@ -8513,27 +8513,27 @@
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -8543,7 +8543,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8897,27 +8897,27 @@
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
@@ -8927,7 +8927,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -8939,12 +8939,12 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C134" t="inlineStr"/>
@@ -8961,27 +8961,27 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -9025,27 +9025,27 @@
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9153,27 +9153,27 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9409,27 +9409,27 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9473,27 +9473,27 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -9537,27 +9537,27 @@
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -9567,7 +9567,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -9601,27 +9601,27 @@
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9771,12 +9771,12 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9921,27 +9921,27 @@
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -10049,27 +10049,27 @@
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10091,12 +10091,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10177,27 +10177,27 @@
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10369,27 +10369,27 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10507,12 +10507,12 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10527,7 +10527,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10640,7 +10640,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10699,12 +10699,12 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>110826062045244</t>
+          <t>110826072522043</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>110826062045384</t>
+          <t>110826062045291</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>110826072521949</t>
+          <t>110826062045244</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>110826072522012</t>
+          <t>110826072521981</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>110826062045291</t>
+          <t>110826072522012</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>110826072521934</t>
+          <t>110826062045259</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>110826072522043</t>
+          <t>110826072521949</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11595,12 +11595,12 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>110826072522028</t>
+          <t>110826072521965</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11659,12 +11659,12 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>110826072521965</t>
+          <t>110826072521934</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>110826072521981</t>
+          <t>110826062045275</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>110826062045259</t>
+          <t>110826062045384</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11856,7 +11856,7 @@
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>110826062045275</t>
+          <t>110826072521996</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11915,12 +11915,12 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>110826072521996</t>
+          <t>110826072522028</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11984,7 +11984,7 @@
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -12048,7 +12048,7 @@
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12171,12 +12171,12 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12235,12 +12235,12 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12299,12 +12299,12 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12464,7 +12464,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12656,7 +12656,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
@@ -12673,22 +12673,22 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12720,7 +12720,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12848,7 +12848,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
@@ -12865,22 +12865,22 @@
       <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -13121,22 +13121,22 @@
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -13185,22 +13185,22 @@
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
@@ -13259,12 +13259,12 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>110826062045525</t>
+          <t>110826062045681</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>110826062045791</t>
+          <t>110826062046400</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>110826062045431</t>
+          <t>110826062045775</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>110826062045541</t>
+          <t>110826062045338</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>110826062045369</t>
+          <t>110826062045416</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>110826062045494</t>
+          <t>110826062045369</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>110826062045509</t>
+          <t>110826062045431</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>110826062045338</t>
+          <t>110826062045400</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>110826062045947</t>
+          <t>110826062045838</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>110826062045775</t>
+          <t>110826062045791</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>110826062045916</t>
+          <t>110826062046338</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>110826062045728</t>
+          <t>110826062045525</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>110826062045416</t>
+          <t>110826062045509</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14091,12 +14091,12 @@
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>110826062045447</t>
+          <t>110826062045353</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14111,7 +14111,7 @@
       </c>
       <c r="M214" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
@@ -14155,12 +14155,12 @@
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>110826062045400</t>
+          <t>110826062045447</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14175,7 +14175,7 @@
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>110826062046400</t>
+          <t>110826062045556</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14288,7 +14288,7 @@
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>110826062046369</t>
+          <t>110826062045884</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>110826062045353</t>
+          <t>110826062046322</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14416,7 +14416,7 @@
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>110826062045853</t>
+          <t>110826062045806</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>110826062046322</t>
+          <t>110826062045322</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14539,12 +14539,12 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>110826062045681</t>
+          <t>110826062046384</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14559,7 +14559,7 @@
       </c>
       <c r="M221" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N221" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>110826062045884</t>
+          <t>110826062045494</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14672,7 +14672,7 @@
       </c>
       <c r="J223" t="inlineStr">
         <is>
-          <t>110826062045869</t>
+          <t>110826062045541</t>
         </is>
       </c>
       <c r="K223" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>110826062045822</t>
+          <t>110826062046353</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>110826062045806</t>
+          <t>110826062045759</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>110826062045838</t>
+          <t>110826062045478</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14928,7 +14928,7 @@
       </c>
       <c r="J227" t="inlineStr">
         <is>
-          <t>110826062045463</t>
+          <t>110826062046369</t>
         </is>
       </c>
       <c r="K227" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>110826062045572</t>
+          <t>110826062045697</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>110826062045322</t>
+          <t>110826062045572</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>110826062046384</t>
+          <t>110826062045463</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>110826062045556</t>
+          <t>110826062045822</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15243,12 +15243,12 @@
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>110826062045306</t>
+          <t>110826062045869</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15263,7 +15263,7 @@
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N232" t="inlineStr">
@@ -15312,7 +15312,7 @@
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>110826062045478</t>
+          <t>110826062045728</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>110826062045759</t>
+          <t>110826062045853</t>
         </is>
       </c>
       <c r="K234" t="inlineStr">
@@ -15408,39 +15408,39 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C235" t="inlineStr"/>
       <c r="D235" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101P-1      </t>
+          <t xml:space="preserve">INO102-1       </t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
         </is>
       </c>
       <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>110826062045697</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15455,7 +15455,7 @@
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N235" t="inlineStr">
@@ -15472,39 +15472,39 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C236" t="inlineStr"/>
       <c r="D236" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101P-1      </t>
+          <t xml:space="preserve">INO102-1       </t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>110826062046353</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15519,7 +15519,7 @@
       </c>
       <c r="M236" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N236" t="inlineStr">
@@ -15536,39 +15536,39 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C237" t="inlineStr"/>
       <c r="D237" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101P-1      </t>
+          <t xml:space="preserve">INO102-1       </t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
         </is>
       </c>
       <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>110826062046338</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15583,7 +15583,7 @@
       </c>
       <c r="M237" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N237" t="inlineStr">
@@ -15632,7 +15632,7 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -15728,39 +15728,39 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C240" t="inlineStr"/>
       <c r="D240" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-1       </t>
+          <t xml:space="preserve">INO102-2       </t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
         </is>
       </c>
       <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15775,7 +15775,7 @@
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N240" t="inlineStr">
@@ -15798,33 +15798,33 @@
       <c r="C241" t="inlineStr"/>
       <c r="D241" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-1       </t>
+          <t xml:space="preserve">INO102-2       </t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
         </is>
       </c>
       <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15839,7 +15839,7 @@
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
@@ -15856,39 +15856,39 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C242" t="inlineStr"/>
       <c r="D242" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-1       </t>
+          <t xml:space="preserve">INO103-2       </t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
         </is>
       </c>
       <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>MMQT4</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15903,7 +15903,7 @@
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
@@ -15920,39 +15920,39 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C243" t="inlineStr"/>
       <c r="D243" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-2       </t>
+          <t xml:space="preserve">INO104-1       </t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
         </is>
       </c>
       <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -15967,7 +15967,7 @@
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N243" t="inlineStr">
@@ -15990,33 +15990,33 @@
       <c r="C244" t="inlineStr"/>
       <c r="D244" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-2       </t>
+          <t xml:space="preserve">INO104-1       </t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
         </is>
       </c>
       <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16031,7 +16031,7 @@
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N244" t="inlineStr">
@@ -16048,39 +16048,39 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C245" t="inlineStr"/>
       <c r="D245" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO103-2       </t>
+          <t xml:space="preserve">INO104-1       </t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
         </is>
       </c>
       <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>MMQT4</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16095,7 +16095,7 @@
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
@@ -16118,12 +16118,12 @@
       <c r="C246" t="inlineStr"/>
       <c r="D246" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-1       </t>
+          <t xml:space="preserve">INO104-2       </t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
         </is>
       </c>
       <c r="F246" t="inlineStr"/>
@@ -16139,12 +16139,12 @@
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16159,7 +16159,7 @@
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
@@ -16182,33 +16182,33 @@
       <c r="C247" t="inlineStr"/>
       <c r="D247" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-1       </t>
+          <t xml:space="preserve">INO104-2       </t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
         </is>
       </c>
       <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056680</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -16223,7 +16223,7 @@
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="N247" t="inlineStr">
@@ -16240,39 +16240,39 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C248" t="inlineStr"/>
       <c r="D248" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-1       </t>
+          <t xml:space="preserve">INO104N-1      </t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
+          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
         </is>
       </c>
       <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
@@ -16310,12 +16310,12 @@
       <c r="C249" t="inlineStr"/>
       <c r="D249" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-2       </t>
+          <t xml:space="preserve">INO104N-1      </t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
+          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
         </is>
       </c>
       <c r="F249" t="inlineStr"/>
@@ -16331,12 +16331,12 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>180226073056680</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -16351,7 +16351,7 @@
       </c>
       <c r="M249" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N249" t="inlineStr">
@@ -16368,29 +16368,29 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C250" t="inlineStr"/>
       <c r="D250" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-2       </t>
+          <t xml:space="preserve">INO104N-1      </t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
+          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
         </is>
       </c>
       <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -16400,7 +16400,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -16432,7 +16432,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C251" t="inlineStr"/>
@@ -16449,22 +16449,22 @@
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
@@ -16479,7 +16479,7 @@
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N251" t="inlineStr">
@@ -16624,39 +16624,39 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C254" t="inlineStr"/>
       <c r="D254" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -16671,7 +16671,7 @@
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N254" t="inlineStr">
@@ -16694,12 +16694,12 @@
       <c r="C255" t="inlineStr"/>
       <c r="D255" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F255" t="inlineStr"/>
@@ -16715,12 +16715,12 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
@@ -16752,39 +16752,39 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C256" t="inlineStr"/>
       <c r="D256" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -16799,7 +16799,7 @@
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N256" t="inlineStr">
@@ -16816,39 +16816,39 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C257" t="inlineStr"/>
       <c r="D257" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U1133G         </t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>22/11/2031</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>300</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -16863,7 +16863,7 @@
       </c>
       <c r="M257" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>300</t>
         </is>
       </c>
       <c r="N257" t="inlineStr">
@@ -16880,39 +16880,39 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C258" t="inlineStr"/>
       <c r="D258" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U889-01        </t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
         </is>
       </c>
       <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -16927,7 +16927,7 @@
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N258" t="inlineStr">
@@ -16944,44 +16944,44 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C259" t="inlineStr"/>
       <c r="D259" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U889-01        </t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
         </is>
       </c>
       <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>09/12/2031</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1912</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>180626072347907</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L259" t="inlineStr">
@@ -16991,7 +16991,7 @@
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>50</t>
         </is>
       </c>
       <c r="N259" t="inlineStr">
@@ -17014,28 +17014,28 @@
       <c r="C260" t="inlineStr"/>
       <c r="D260" t="inlineStr">
         <is>
-          <t xml:space="preserve">U1133G         </t>
+          <t xml:space="preserve">U891           </t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
+          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
         </is>
       </c>
       <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
-          <t>22/11/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J260" t="inlineStr">
@@ -17055,7 +17055,7 @@
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N260" t="inlineStr">
@@ -17072,39 +17072,39 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C261" t="inlineStr"/>
       <c r="D261" t="inlineStr">
         <is>
-          <t xml:space="preserve">U889-01        </t>
+          <t xml:space="preserve">U948-1         </t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
+          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
         </is>
       </c>
       <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>31/01/2032</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>507</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>100826061846740</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17119,202 +17119,10 @@
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>507</t>
         </is>
       </c>
       <c r="N261" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t>CAL-001-001-001</t>
-        </is>
-      </c>
-      <c r="C262" t="inlineStr"/>
-      <c r="D262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U889-01        </t>
-        </is>
-      </c>
-      <c r="E262" t="inlineStr">
-        <is>
-          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
-        </is>
-      </c>
-      <c r="F262" t="inlineStr"/>
-      <c r="G262" t="inlineStr">
-        <is>
-          <t>09/12/2031</t>
-        </is>
-      </c>
-      <c r="H262" t="inlineStr">
-        <is>
-          <t>1912</t>
-        </is>
-      </c>
-      <c r="I262" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="J262" t="inlineStr">
-        <is>
-          <t>180626072347907</t>
-        </is>
-      </c>
-      <c r="K262" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="L262" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M262" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="N262" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B263" t="inlineStr">
-        <is>
-          <t>CAL-027-008-001</t>
-        </is>
-      </c>
-      <c r="C263" t="inlineStr"/>
-      <c r="D263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U891           </t>
-        </is>
-      </c>
-      <c r="E263" t="inlineStr">
-        <is>
-          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
-        </is>
-      </c>
-      <c r="F263" t="inlineStr"/>
-      <c r="G263" t="inlineStr">
-        <is>
-          <t>03/11/2031</t>
-        </is>
-      </c>
-      <c r="H263" t="inlineStr">
-        <is>
-          <t>1876</t>
-        </is>
-      </c>
-      <c r="I263" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="J263" t="inlineStr">
-        <is>
-          <t>110226132440294</t>
-        </is>
-      </c>
-      <c r="K263" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L263" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M263" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="N263" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>CAL-001-001-001</t>
-        </is>
-      </c>
-      <c r="C264" t="inlineStr"/>
-      <c r="D264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U948-1         </t>
-        </is>
-      </c>
-      <c r="E264" t="inlineStr">
-        <is>
-          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
-        </is>
-      </c>
-      <c r="F264" t="inlineStr"/>
-      <c r="G264" t="inlineStr">
-        <is>
-          <t>31/01/2032</t>
-        </is>
-      </c>
-      <c r="H264" t="inlineStr">
-        <is>
-          <t>1965</t>
-        </is>
-      </c>
-      <c r="I264" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="J264" t="inlineStr">
-        <is>
-          <t>100826061846740</t>
-        </is>
-      </c>
-      <c r="K264" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L264" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M264" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="N264" t="inlineStr">
         <is>
           <t>NO</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/09/2026 09:31:04
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,22 +513,22 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -779,12 +779,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2187,12 +2187,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2443,12 +2443,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-027-006-002</t>
+          <t>CAL-027-007-002</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2635,12 +2635,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>280826111844285</t>
+          <t>280826060740757</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-027-007-002</t>
+          <t>CAL-027-006-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2699,12 +2699,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>48</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>280826060740757</t>
+          <t>280826111844285</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>48</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2881,22 +2881,22 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2945,22 +2945,22 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3137,22 +3137,22 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4801,22 +4801,22 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4865,12 +4865,12 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4929,12 +4929,12 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5185,12 +5185,12 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5249,12 +5249,12 @@
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5313,12 +5313,12 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5377,22 +5377,22 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5441,12 +5441,12 @@
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5505,12 +5505,12 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5761,12 +5761,12 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5889,12 +5889,12 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,12 +6081,12 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6379,12 +6379,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6475,12 +6475,12 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6507,12 +6507,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6571,12 +6571,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6699,12 +6699,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -6731,12 +6731,12 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6827,12 +6827,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C101" t="inlineStr"/>
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6891,12 +6891,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C102" t="inlineStr"/>
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7169,27 +7169,27 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -7233,27 +7233,27 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7361,27 +7361,27 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,22 +7489,22 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7553,27 +7553,27 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7617,27 +7617,27 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7873,27 +7873,27 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7947,12 +7947,12 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8011,12 +8011,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -8065,27 +8065,27 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -8129,27 +8129,27 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8193,27 +8193,27 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8321,27 +8321,27 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8400,12 +8400,12 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -8449,27 +8449,27 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8577,27 +8577,27 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8641,27 +8641,27 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8705,27 +8705,27 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8833,27 +8833,27 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -8897,27 +8897,27 @@
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
@@ -8927,7 +8927,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9131,12 +9131,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
@@ -9153,27 +9153,27 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9195,12 +9195,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
@@ -9217,27 +9217,27 @@
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -9247,7 +9247,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9451,12 +9451,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9579,12 +9579,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9793,27 +9793,27 @@
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -10049,27 +10049,27 @@
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10113,27 +10113,27 @@
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -10177,27 +10177,27 @@
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -10241,27 +10241,27 @@
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10305,27 +10305,27 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10384,7 +10384,7 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10507,12 +10507,12 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10527,7 +10527,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -10640,7 +10640,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10699,12 +10699,12 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>110826072521981</t>
+          <t>110826072522028</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>110826072521949</t>
+          <t>110826072522043</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>110826062045275</t>
+          <t>110826072521981</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>110826072522012</t>
+          <t>110826062045275</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>110826062045384</t>
+          <t>110826072522012</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>110826072522028</t>
+          <t>110826072521949</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>110826062045291</t>
+          <t>110826072521965</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>110826062045259</t>
+          <t>110826062045384</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>110826072521996</t>
+          <t>110826062045259</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>110826072522043</t>
+          <t>110826072521996</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>110826072521965</t>
+          <t>110826062045291</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12171,12 +12171,12 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12240,7 +12240,7 @@
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12304,7 +12304,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12363,12 +12363,12 @@
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12464,7 +12464,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12720,7 +12720,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -12939,12 +12939,12 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
@@ -12993,22 +12993,22 @@
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
@@ -13057,22 +13057,22 @@
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13087,7 +13087,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>110826062045416</t>
+          <t>110826062045509</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>110826062045697</t>
+          <t>110826062045369</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>110826062045775</t>
+          <t>110826062045338</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>110826062045509</t>
+          <t>110826062045759</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>110826062045338</t>
+          <t>110826062045697</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13451,12 +13451,12 @@
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>110826062045681</t>
+          <t>110826062045775</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
@@ -13515,12 +13515,12 @@
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>110826062045759</t>
+          <t>110826062045681</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13535,7 +13535,7 @@
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N205" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>110826062045463</t>
+          <t>110826062045416</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -13648,7 +13648,7 @@
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>110826062045369</t>
+          <t>110826062046400</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13712,7 +13712,7 @@
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>110826062045431</t>
+          <t>110826062045791</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13776,7 +13776,7 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>110826062045791</t>
+          <t>110826062045463</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13840,7 +13840,7 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>110826062045525</t>
+          <t>110826062045431</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>110826062045541</t>
+          <t>110826062045525</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13968,7 +13968,7 @@
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>110826062045400</t>
+          <t>110826062045353</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -14027,12 +14027,12 @@
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>110826062045822</t>
+          <t>110826062045447</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14047,7 +14047,7 @@
       </c>
       <c r="M213" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N213" t="inlineStr">
@@ -14096,7 +14096,7 @@
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>110826062045572</t>
+          <t>110826062046322</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14160,7 +14160,7 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>110826062045478</t>
+          <t>110826062045556</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>110826062046400</t>
+          <t>110826062045806</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>110826062045806</t>
+          <t>110826062045478</t>
         </is>
       </c>
       <c r="K218" t="inlineStr">
@@ -14411,12 +14411,12 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>110826062045447</t>
+          <t>110826062045494</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14431,7 +14431,7 @@
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N219" t="inlineStr">
@@ -14480,7 +14480,7 @@
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>110826062045494</t>
+          <t>110826062045541</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="J221" t="inlineStr">
         <is>
-          <t>110826062045838</t>
+          <t>110826062045572</t>
         </is>
       </c>
       <c r="K221" t="inlineStr">
@@ -14608,7 +14608,7 @@
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>110826062045353</t>
+          <t>110826062045728</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>110826062046322</t>
+          <t>110826062045822</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>110826062045728</t>
+          <t>110826062045838</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>110826062045556</t>
+          <t>110826062045400</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14987,12 +14987,12 @@
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -15007,7 +15007,7 @@
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N228" t="inlineStr">
@@ -15051,12 +15051,12 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -15071,7 +15071,7 @@
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N229" t="inlineStr">
@@ -15115,12 +15115,12 @@
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
@@ -15135,7 +15135,7 @@
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N230" t="inlineStr">
@@ -15179,12 +15179,12 @@
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J231" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">
@@ -15199,7 +15199,7 @@
       </c>
       <c r="M231" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N231" t="inlineStr">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C232" t="inlineStr"/>
@@ -15243,12 +15243,12 @@
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15263,7 +15263,7 @@
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N232" t="inlineStr">
@@ -15280,7 +15280,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C233" t="inlineStr"/>
@@ -15307,12 +15307,12 @@
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J233" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K233" t="inlineStr">
@@ -15327,7 +15327,7 @@
       </c>
       <c r="M233" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N233" t="inlineStr">
@@ -15435,12 +15435,12 @@
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K235" t="inlineStr">
@@ -15455,7 +15455,7 @@
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N235" t="inlineStr">
@@ -15489,22 +15489,22 @@
       <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J236" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -15519,7 +15519,7 @@
       </c>
       <c r="M236" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N236" t="inlineStr">
@@ -15553,22 +15553,22 @@
       <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15583,7 +15583,7 @@
       </c>
       <c r="M237" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N237" t="inlineStr">
@@ -15728,7 +15728,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C240" t="inlineStr"/>
@@ -15745,22 +15745,22 @@
       <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K240" t="inlineStr">
@@ -15775,7 +15775,7 @@
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N240" t="inlineStr">
@@ -15792,7 +15792,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C241" t="inlineStr"/>
@@ -15809,22 +15809,22 @@
       <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K241" t="inlineStr">
@@ -15839,7 +15839,7 @@
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
@@ -15856,7 +15856,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C242" t="inlineStr"/>
@@ -15873,22 +15873,22 @@
       <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K242" t="inlineStr">
@@ -15903,7 +15903,7 @@
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
@@ -15920,7 +15920,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C243" t="inlineStr"/>
@@ -15937,22 +15937,22 @@
       <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -15967,7 +15967,7 @@
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N243" t="inlineStr">
@@ -15984,7 +15984,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C244" t="inlineStr"/>
@@ -16001,22 +16001,22 @@
       <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16031,7 +16031,7 @@
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N244" t="inlineStr">
@@ -16048,7 +16048,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C245" t="inlineStr"/>
@@ -16065,22 +16065,22 @@
       <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -16095,7 +16095,7 @@
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
@@ -16112,7 +16112,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C246" t="inlineStr"/>
@@ -16129,22 +16129,22 @@
       <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K246" t="inlineStr">
@@ -16159,7 +16159,7 @@
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
@@ -16240,7 +16240,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C248" t="inlineStr"/>
@@ -16257,22 +16257,22 @@
       <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
@@ -16368,7 +16368,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C250" t="inlineStr"/>
@@ -16385,27 +16385,27 @@
       <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
-          <t>09/12/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>1912</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>180626072347907</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L250" t="inlineStr">
@@ -16415,7 +16415,7 @@
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N250" t="inlineStr">
@@ -16432,7 +16432,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C251" t="inlineStr"/>
@@ -16449,27 +16449,27 @@
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>09/12/2031</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1912</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J251" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>180626072347907</t>
         </is>
       </c>
       <c r="K251" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L251" t="inlineStr">
@@ -16479,7 +16479,7 @@
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="N251" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/09/2026 13:06:48
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N227"/>
+  <dimension ref="A1:N226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,12 +513,12 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -720,7 +720,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -779,12 +779,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1003,12 +1003,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1995,12 +1995,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2315,12 +2315,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2817,22 +2817,22 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3009,22 +3009,22 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519104</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>320</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3137,22 +3137,22 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-006-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -3531,12 +3531,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104519104</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>320</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CAL-026-006-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3585,22 +3585,22 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4929,22 +4929,22 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,12 +5057,12 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5185,22 +5185,22 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5249,12 +5249,12 @@
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5313,12 +5313,12 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5377,12 +5377,12 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5451,12 +5451,12 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5505,12 +5505,12 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5569,12 +5569,12 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5697,12 +5697,12 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5761,12 +5761,12 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5825,22 +5825,22 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5953,12 +5953,12 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6017,12 +6017,12 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6187,12 +6187,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6251,12 +6251,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C92" t="inlineStr"/>
@@ -6283,12 +6283,12 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -6315,12 +6315,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6379,12 +6379,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6411,12 +6411,12 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6507,12 +6507,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6635,12 +6635,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6864,7 +6864,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7041,27 +7041,27 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7169,27 +7169,27 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -7233,27 +7233,27 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,27 +7361,27 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7425,27 +7425,27 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7489,27 +7489,27 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7681,27 +7681,27 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7873,27 +7873,27 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7937,22 +7937,22 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8257,22 +8257,22 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8449,27 +8449,27 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8705,27 +8705,27 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8961,27 +8961,27 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -9003,12 +9003,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9089,27 +9089,27 @@
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -9119,7 +9119,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9217,27 +9217,27 @@
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -9247,7 +9247,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -9281,27 +9281,27 @@
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9409,27 +9409,27 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9473,27 +9473,27 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9665,27 +9665,27 @@
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -9707,12 +9707,12 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
@@ -9729,27 +9729,27 @@
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -9985,27 +9985,27 @@
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10091,12 +10091,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10241,27 +10241,27 @@
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10369,27 +10369,27 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10635,12 +10635,12 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -10699,12 +10699,12 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>110826072521981</t>
+          <t>110826072522012</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>110826072521996</t>
+          <t>110826062045275</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>110826062045259</t>
+          <t>110826072521996</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11339,12 +11339,12 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>110826072522028</t>
+          <t>110826062045291</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>110826072522012</t>
+          <t>110826072521965</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>110826062045275</t>
+          <t>110826062045384</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>110826072521949</t>
+          <t>110826062045259</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>110826062045384</t>
+          <t>110826072521949</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11659,12 +11659,12 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>110826062045291</t>
+          <t>110826072522028</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11728,7 +11728,7 @@
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>110826072521965</t>
+          <t>110826072522043</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11792,7 +11792,7 @@
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>110826072522043</t>
+          <t>110826072521981</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12107,12 +12107,12 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12171,12 +12171,12 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -12939,12 +12939,12 @@
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>110826062045353</t>
+          <t>110826062045431</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13168,39 +13168,39 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101P-1      </t>
+          <t xml:space="preserve">INO102-1       </t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>110826062045431</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
@@ -13259,12 +13259,12 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
@@ -13313,22 +13313,22 @@
       <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13343,7 +13343,7 @@
       </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N202" t="inlineStr">
@@ -13387,12 +13387,12 @@
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13407,7 +13407,7 @@
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N203" t="inlineStr">
@@ -13441,22 +13441,22 @@
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
@@ -13488,39 +13488,39 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-1       </t>
+          <t xml:space="preserve">INO102-2       </t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
         </is>
       </c>
       <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13535,7 +13535,7 @@
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N205" t="inlineStr">
@@ -13616,39 +13616,39 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-2       </t>
+          <t xml:space="preserve">INO103-2       </t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
         </is>
       </c>
       <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>MMQT4</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N207" t="inlineStr">
@@ -13680,39 +13680,39 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO103-2       </t>
+          <t xml:space="preserve">INO104-1       </t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
         </is>
       </c>
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>MMQT4</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13727,7 +13727,7 @@
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N208" t="inlineStr">
@@ -13835,12 +13835,12 @@
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13855,7 +13855,7 @@
       </c>
       <c r="M210" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N210" t="inlineStr">
@@ -13878,12 +13878,12 @@
       <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-1       </t>
+          <t xml:space="preserve">INO104-2       </t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
         </is>
       </c>
       <c r="F211" t="inlineStr"/>
@@ -13904,7 +13904,7 @@
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13953,22 +13953,22 @@
       <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056680</t>
         </is>
       </c>
       <c r="K212" t="inlineStr">
@@ -13983,7 +13983,7 @@
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
@@ -14000,39 +14000,39 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C213" t="inlineStr"/>
       <c r="D213" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-2       </t>
+          <t xml:space="preserve">INO104N-1      </t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
+          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
         </is>
       </c>
       <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>180226073056680</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K213" t="inlineStr">
@@ -14047,7 +14047,7 @@
       </c>
       <c r="M213" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N213" t="inlineStr">
@@ -14081,22 +14081,22 @@
       <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -14111,7 +14111,7 @@
       </c>
       <c r="M214" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
@@ -14128,7 +14128,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C215" t="inlineStr"/>
@@ -14145,22 +14145,22 @@
       <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14175,7 +14175,7 @@
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
@@ -14209,22 +14209,22 @@
       <c r="F216" t="inlineStr"/>
       <c r="G216" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K216" t="inlineStr">
@@ -14239,7 +14239,7 @@
       </c>
       <c r="M216" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
@@ -14256,7 +14256,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C217" t="inlineStr"/>
@@ -14273,22 +14273,22 @@
       <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>280726145222119</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
@@ -14303,7 +14303,7 @@
       </c>
       <c r="M217" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N217" t="inlineStr">
@@ -14390,12 +14390,12 @@
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F219" t="inlineStr"/>
@@ -14411,12 +14411,12 @@
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K219" t="inlineStr">
@@ -14431,7 +14431,7 @@
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N219" t="inlineStr">
@@ -14448,7 +14448,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C220" t="inlineStr"/>
@@ -14465,22 +14465,22 @@
       <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J220" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K220" t="inlineStr">
@@ -14495,7 +14495,7 @@
       </c>
       <c r="M220" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N220" t="inlineStr">
@@ -14576,39 +14576,39 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C222" t="inlineStr"/>
       <c r="D222" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U1133G         </t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
         </is>
       </c>
       <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>22/11/2031</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>300</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K222" t="inlineStr">
@@ -14623,7 +14623,7 @@
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>300</t>
         </is>
       </c>
       <c r="N222" t="inlineStr">
@@ -14646,28 +14646,28 @@
       <c r="C223" t="inlineStr"/>
       <c r="D223" t="inlineStr">
         <is>
-          <t xml:space="preserve">U1133G         </t>
+          <t xml:space="preserve">U889-01        </t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
+          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
         </is>
       </c>
       <c r="F223" t="inlineStr"/>
       <c r="G223" t="inlineStr">
         <is>
-          <t>22/11/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J223" t="inlineStr">
@@ -14687,7 +14687,7 @@
       </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N223" t="inlineStr">
@@ -14704,7 +14704,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C224" t="inlineStr"/>
@@ -14721,27 +14721,27 @@
       <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>09/12/2031</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1912</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>180626072347907</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L224" t="inlineStr">
@@ -14751,7 +14751,7 @@
       </c>
       <c r="M224" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="N224" t="inlineStr">
@@ -14768,44 +14768,44 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C225" t="inlineStr"/>
       <c r="D225" t="inlineStr">
         <is>
-          <t xml:space="preserve">U889-01        </t>
+          <t xml:space="preserve">U891           </t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
+          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
         </is>
       </c>
       <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr">
         <is>
-          <t>09/12/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>1912</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J225" t="inlineStr">
         <is>
-          <t>180626072347907</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K225" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L225" t="inlineStr">
@@ -14815,7 +14815,7 @@
       </c>
       <c r="M225" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N225" t="inlineStr">
@@ -14832,39 +14832,39 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C226" t="inlineStr"/>
       <c r="D226" t="inlineStr">
         <is>
-          <t xml:space="preserve">U891           </t>
+          <t xml:space="preserve">U948-1         </t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
+          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
         </is>
       </c>
       <c r="F226" t="inlineStr"/>
       <c r="G226" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>31/01/2032</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>507</t>
         </is>
       </c>
       <c r="J226" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>100826061846740</t>
         </is>
       </c>
       <c r="K226" t="inlineStr">
@@ -14879,74 +14879,10 @@
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>507</t>
         </is>
       </c>
       <c r="N226" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>CAL-001-001-001</t>
-        </is>
-      </c>
-      <c r="C227" t="inlineStr"/>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U948-1         </t>
-        </is>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
-        </is>
-      </c>
-      <c r="F227" t="inlineStr"/>
-      <c r="G227" t="inlineStr">
-        <is>
-          <t>31/01/2032</t>
-        </is>
-      </c>
-      <c r="H227" t="inlineStr">
-        <is>
-          <t>1965</t>
-        </is>
-      </c>
-      <c r="I227" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="J227" t="inlineStr">
-        <is>
-          <t>100826061846740</t>
-        </is>
-      </c>
-      <c r="K227" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L227" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M227" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="N227" t="inlineStr">
         <is>
           <t>NO</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/09/2026 14:13:32
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N216"/>
+  <dimension ref="A1:N215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,22 +513,22 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1940</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1035,12 +1035,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1995,12 +1995,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2753,22 +2753,22 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519026</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2817,22 +2817,22 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2881,22 +2881,22 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2945,22 +2945,22 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3009,22 +3009,22 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>110226132439732</t>
+          <t>130526104519026</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-006-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3137,22 +3137,22 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -3521,22 +3521,22 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CAL-026-006-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -3585,22 +3585,22 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -3649,22 +3649,22 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439732</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439622</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -3777,22 +3777,22 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132439622</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4545,12 +4545,12 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4747,12 +4747,12 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4865,12 +4865,12 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5451,12 +5451,12 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5569,12 +5569,12 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5633,22 +5633,22 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5697,12 +5697,12 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5953,12 +5953,12 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6017,12 +6017,12 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,22 +6081,22 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6187,12 +6187,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6411,12 +6411,12 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6443,12 +6443,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6507,12 +6507,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6571,12 +6571,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6635,12 +6635,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6699,12 +6699,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6827,12 +6827,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C101" t="inlineStr"/>
@@ -6859,12 +6859,12 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6891,12 +6891,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C102" t="inlineStr"/>
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7169,27 +7169,27 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -7233,27 +7233,27 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7297,27 +7297,27 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7489,22 +7489,22 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7627,12 +7627,12 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7809,27 +7809,27 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -7873,27 +7873,27 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7937,27 +7937,27 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8001,22 +8001,22 @@
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -8065,27 +8065,27 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8193,27 +8193,27 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8321,27 +8321,27 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8961,27 +8961,27 @@
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9067,12 +9067,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C136" t="inlineStr"/>
@@ -9089,27 +9089,27 @@
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -9119,7 +9119,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9217,27 +9217,27 @@
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -9247,7 +9247,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9323,12 +9323,12 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9473,27 +9473,27 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -9515,12 +9515,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
@@ -9537,27 +9537,27 @@
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -9567,7 +9567,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -9601,27 +9601,27 @@
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9729,27 +9729,27 @@
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10113,27 +10113,27 @@
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1897</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
@@ -10143,7 +10143,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10305,27 +10305,27 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10369,27 +10369,27 @@
       <c r="F156" t="inlineStr"/>
       <c r="G156" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10640,7 +10640,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -11120,29 +11120,29 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr">
         <is>
-          <t xml:space="preserve">BID101P-3      </t>
+          <t xml:space="preserve">BID102-1       </t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t xml:space="preserve">BIDE 3 AGUJEROS BLANCO LINEA ACQUA PLUS                               </t>
+          <t xml:space="preserve">BIDE 1 AGUJERO BLANCO LINEA LOFT                                      </t>
         </is>
       </c>
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11152,7 +11152,7 @@
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>110826072521949</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11216,7 +11216,7 @@
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11254,33 +11254,33 @@
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr">
         <is>
-          <t xml:space="preserve">BID102-1       </t>
+          <t xml:space="preserve">BID102-3       </t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t xml:space="preserve">BIDE 1 AGUJERO BLANCO LINEA LOFT                                      </t>
+          <t xml:space="preserve">BIDE 3 AGUJEROS BLANCO LINEA LOFT                                     </t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/02/2032</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1984</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226070819834</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11318,33 +11318,33 @@
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr">
         <is>
-          <t xml:space="preserve">BID102-3       </t>
+          <t xml:space="preserve">BID104-1       </t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t xml:space="preserve">BIDE 3 AGUJEROS BLANCO LINEA LOFT                                     </t>
+          <t xml:space="preserve">BIDE 1 AGUJERO BLANCO LINEA STONE                                     </t>
         </is>
       </c>
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>19/02/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>200226070819834</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11510,12 +11510,12 @@
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
-          <t xml:space="preserve">BID104-1       </t>
+          <t xml:space="preserve">BID104-3       </t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t xml:space="preserve">BIDE 1 AGUJERO BLANCO LINEA STONE                                     </t>
+          <t xml:space="preserve">BIDE 3 AGUJEROS BLANCO LINEA STONE                                    </t>
         </is>
       </c>
       <c r="F174" t="inlineStr"/>
@@ -11531,12 +11531,12 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11632,39 +11632,39 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
-          <t xml:space="preserve">BID104-3       </t>
+          <t xml:space="preserve">BID104N-1      </t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t xml:space="preserve">BIDE 3 AGUJEROS BLANCO LINEA STONE                                    </t>
+          <t xml:space="preserve">BIDE 1 AGUJERO BLACK LINEA STONE                                      </t>
         </is>
       </c>
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11723,12 +11723,12 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11841,22 +11841,22 @@
       <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11888,39 +11888,39 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
-          <t xml:space="preserve">BID104N-1      </t>
+          <t xml:space="preserve">BID104N-3      </t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t xml:space="preserve">BIDE 1 AGUJERO BLACK LINEA STONE                                      </t>
+          <t xml:space="preserve">BIDE 3 AGUJEROS BLACK LINEA STONE                                     </t>
         </is>
       </c>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11979,12 +11979,12 @@
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12075,44 +12075,44 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr">
         <is>
-          <t xml:space="preserve">BID104N-3      </t>
+          <t xml:space="preserve">G030           </t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t xml:space="preserve">BIDE 3 AGUJEROS BLACK LINEA STONE                                     </t>
+          <t xml:space="preserve">NIPLE IZQUIERDO P/TUERCA DE CONEXION                                  </t>
         </is>
       </c>
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>17280</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>060226143406794</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>17280</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12139,44 +12139,44 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
-          <t xml:space="preserve">G030           </t>
+          <t xml:space="preserve">INO101-1       </t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIPLE IZQUIERDO P/TUERCA DE CONEXION                                  </t>
+          <t>INO101-1 - INODORO BLANCO C/ASIENTO LINEA ACQUA</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>17280</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>060226143406794</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>17280</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12235,12 +12235,12 @@
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12278,33 +12278,33 @@
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101-1       </t>
+          <t xml:space="preserve">INO101-2       </t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>INO101-1 - INODORO BLANCO C/ASIENTO LINEA ACQUA</t>
+          <t>INO101-2 - DEPOSITO C/DESCARGA DUAL BLANCO LINEA ACQUA</t>
         </is>
       </c>
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12400,39 +12400,39 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101-2       </t>
+          <t xml:space="preserve">INO101P-1      </t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>INO101-2 - DEPOSITO C/DESCARGA DUAL BLANCO LINEA ACQUA</t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
         </is>
       </c>
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>01/02/2032</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1966</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>110826062045431</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12464,39 +12464,39 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101P-1      </t>
+          <t xml:space="preserve">INO102-1       </t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
         </is>
       </c>
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>110826062045431</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12560,7 +12560,7 @@
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12683,12 +12683,12 @@
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1924</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12784,39 +12784,39 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-1       </t>
+          <t xml:space="preserve">INO102-2       </t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12848,7 +12848,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -12912,39 +12912,39 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-2       </t>
+          <t xml:space="preserve">INO103-2       </t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
         </is>
       </c>
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>MMQT4</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
@@ -12976,39 +12976,39 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO103-2       </t>
+          <t xml:space="preserve">INO104-1       </t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>MMQT4</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
@@ -13057,22 +13057,22 @@
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13087,7 +13087,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
@@ -13131,12 +13131,12 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -13174,12 +13174,12 @@
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-1       </t>
+          <t xml:space="preserve">INO104-2       </t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
@@ -13200,7 +13200,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13249,22 +13249,22 @@
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056680</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
@@ -13296,39 +13296,39 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-2       </t>
+          <t xml:space="preserve">INO104N-1      </t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
+          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
         </is>
       </c>
       <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>180226073056680</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13343,7 +13343,7 @@
       </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N202" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -13377,22 +13377,22 @@
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13407,7 +13407,7 @@
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N203" t="inlineStr">
@@ -13488,7 +13488,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C205" t="inlineStr"/>
@@ -13505,22 +13505,22 @@
       <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1794</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13535,7 +13535,7 @@
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N205" t="inlineStr">
@@ -13680,39 +13680,39 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1952</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>33</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>280726145222384</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
@@ -13727,7 +13727,7 @@
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>33</t>
         </is>
       </c>
       <c r="N208" t="inlineStr">
@@ -13744,7 +13744,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C209" t="inlineStr"/>
@@ -13761,22 +13761,22 @@
       <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
@@ -13791,7 +13791,7 @@
       </c>
       <c r="M209" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N209" t="inlineStr">
@@ -13808,7 +13808,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C210" t="inlineStr"/>
@@ -13825,22 +13825,22 @@
       <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1862</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
@@ -13855,7 +13855,7 @@
       </c>
       <c r="M210" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N210" t="inlineStr">
@@ -13872,39 +13872,39 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U1133G         </t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
         </is>
       </c>
       <c r="F211" t="inlineStr"/>
       <c r="G211" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>22/11/2031</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>300</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
@@ -13919,7 +13919,7 @@
       </c>
       <c r="M211" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>300</t>
         </is>
       </c>
       <c r="N211" t="inlineStr">
@@ -13942,28 +13942,28 @@
       <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr">
         <is>
-          <t xml:space="preserve">U1133G         </t>
+          <t xml:space="preserve">U889-01        </t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
+          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
         </is>
       </c>
       <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr">
         <is>
-          <t>22/11/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1876</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
@@ -13983,7 +13983,7 @@
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
@@ -14070,12 +14070,12 @@
       <c r="C214" t="inlineStr"/>
       <c r="D214" t="inlineStr">
         <is>
-          <t xml:space="preserve">U889-01        </t>
+          <t xml:space="preserve">U891           </t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
+          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
         </is>
       </c>
       <c r="F214" t="inlineStr"/>
@@ -14091,7 +14091,7 @@
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -14111,7 +14111,7 @@
       </c>
       <c r="M214" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
@@ -14128,39 +14128,39 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="inlineStr">
         <is>
-          <t xml:space="preserve">U891           </t>
+          <t xml:space="preserve">U948-1         </t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
+          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
         </is>
       </c>
       <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>31/01/2032</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>507</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>100826061846740</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -14175,74 +14175,10 @@
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>507</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>CAL-001-001-001</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr"/>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U948-1         </t>
-        </is>
-      </c>
-      <c r="E216" t="inlineStr">
-        <is>
-          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
-        </is>
-      </c>
-      <c r="F216" t="inlineStr"/>
-      <c r="G216" t="inlineStr">
-        <is>
-          <t>31/01/2032</t>
-        </is>
-      </c>
-      <c r="H216" t="inlineStr">
-        <is>
-          <t>1965</t>
-        </is>
-      </c>
-      <c r="I216" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="J216" t="inlineStr">
-        <is>
-          <t>100826061846740</t>
-        </is>
-      </c>
-      <c r="K216" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L216" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M216" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="N216" t="inlineStr">
         <is>
           <t>NO</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 14/09/2026 15:46:58
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 15/09/2026 06:02:49
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1939</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1939</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1939</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1940</t>
+          <t>1939</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1815</t>
+          <t>1814</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1848</t>
+          <t>1847</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1919</t>
+          <t>1918</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1919</t>
+          <t>1918</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1897</t>
+          <t>1896</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1846</t>
+          <t>1845</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1891</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1891</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1966</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1924</t>
+          <t>1923</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1794</t>
+          <t>1793</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1952</t>
+          <t>1951</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13766,7 +13766,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>1862</t>
+          <t>1861</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -13958,7 +13958,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1912</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -14086,7 +14086,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>1876</t>
+          <t>1875</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>1965</t>
+          <t>1964</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 16/09/2026 06:05:41
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1939</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1939</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1939</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1939</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1814</t>
+          <t>1813</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1949</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1949</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1949</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1847</t>
+          <t>1846</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1918</t>
+          <t>1917</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1918</t>
+          <t>1917</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1776</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1776</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1896</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1845</t>
+          <t>1844</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1923</t>
+          <t>1922</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1965</t>
+          <t>1964</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1923</t>
+          <t>1922</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1793</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1951</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1861</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13766,7 +13766,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1875</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>1964</t>
+          <t>1963</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 16/09/2026 06:32:45
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N210"/>
+  <dimension ref="A1:N208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -683,12 +683,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -705,22 +705,22 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2753,22 +2753,22 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2945,22 +2945,22 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-026-006-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3009,22 +3009,22 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3329,22 +3329,22 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3393,22 +3393,22 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CAL-026-006-001</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3457,22 +3457,22 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -4097,12 +4097,12 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,12 +4289,12 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4417,12 +4417,12 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4481,12 +4481,12 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4673,22 +4673,22 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4865,12 +4865,12 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,12 +5057,12 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5131,12 +5131,12 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5249,12 +5249,12 @@
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5377,12 +5377,12 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5569,22 +5569,22 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5633,12 +5633,12 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5771,12 +5771,12 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5825,12 +5825,12 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5867,12 +5867,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6027,12 +6027,12 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6123,12 +6123,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6315,12 +6315,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6379,12 +6379,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6507,12 +6507,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -6539,12 +6539,12 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6559,7 +6559,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -6571,12 +6571,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6721,27 +6721,27 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6785,27 +6785,27 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -6849,27 +6849,27 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6913,27 +6913,27 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7179,12 +7179,12 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -7233,27 +7233,27 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7425,27 +7425,27 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7489,27 +7489,27 @@
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7617,22 +7617,22 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7745,27 +7745,27 @@
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -7809,27 +7809,27 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -7888,12 +7888,12 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8065,27 +8065,27 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -8129,27 +8129,27 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8193,27 +8193,27 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8321,27 +8321,27 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8513,27 +8513,27 @@
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -8543,7 +8543,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -8577,27 +8577,27 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8641,27 +8641,27 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8683,12 +8683,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8833,27 +8833,27 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -9003,12 +9003,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -9025,27 +9025,27 @@
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -9067,12 +9067,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C136" t="inlineStr"/>
@@ -9089,27 +9089,27 @@
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -9119,7 +9119,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N136" t="inlineStr">
@@ -9153,27 +9153,27 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9281,27 +9281,27 @@
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -9345,27 +9345,27 @@
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -9375,7 +9375,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -9409,27 +9409,27 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9451,12 +9451,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9537,27 +9537,27 @@
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -9567,7 +9567,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9921,27 +9921,27 @@
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -9985,27 +9985,27 @@
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10192,7 +10192,7 @@
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10251,12 +10251,12 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -11019,12 +11019,12 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11457,22 +11457,22 @@
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11713,22 +11713,22 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1922</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12240,7 +12240,7 @@
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12299,12 +12299,12 @@
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1922</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12993,22 +12993,22 @@
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
@@ -13057,22 +13057,22 @@
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>280726145222119</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13087,7 +13087,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
@@ -13104,7 +13104,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
@@ -13121,22 +13121,22 @@
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -13168,7 +13168,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
@@ -13185,22 +13185,22 @@
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
@@ -13232,7 +13232,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C201" t="inlineStr"/>
@@ -13249,22 +13249,22 @@
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13279,7 +13279,7 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
@@ -13296,39 +13296,39 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13343,7 +13343,7 @@
       </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N202" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -13377,22 +13377,22 @@
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>280726145222384</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13407,7 +13407,7 @@
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N203" t="inlineStr">
@@ -13424,39 +13424,39 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U1133G         </t>
         </is>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
         </is>
       </c>
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>22/11/2031</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>300</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>300</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
@@ -13488,39 +13488,39 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U889-01        </t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
         </is>
       </c>
       <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13535,7 +13535,7 @@
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N205" t="inlineStr">
@@ -13552,44 +13552,44 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
         <is>
-          <t xml:space="preserve">U1133G         </t>
+          <t xml:space="preserve">U889-01        </t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
+          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
         </is>
       </c>
       <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
-          <t>22/11/2031</t>
+          <t>09/12/2031</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>180626072347907</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L206" t="inlineStr">
@@ -13599,7 +13599,7 @@
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>50</t>
         </is>
       </c>
       <c r="N206" t="inlineStr">
@@ -13622,12 +13622,12 @@
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr">
         <is>
-          <t xml:space="preserve">U889-01        </t>
+          <t xml:space="preserve">U891           </t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
+          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
         </is>
       </c>
       <c r="F207" t="inlineStr"/>
@@ -13643,7 +13643,7 @@
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N207" t="inlineStr">
@@ -13686,38 +13686,38 @@
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
-          <t xml:space="preserve">U889-01        </t>
+          <t xml:space="preserve">U948-1         </t>
         </is>
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
+          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
         </is>
       </c>
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
-          <t>09/12/2031</t>
+          <t>31/01/2032</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1963</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>507</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>180626072347907</t>
+          <t>100826061846740</t>
         </is>
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L208" t="inlineStr">
@@ -13727,138 +13727,10 @@
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>507</t>
         </is>
       </c>
       <c r="N208" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>CAL-027-008-001</t>
-        </is>
-      </c>
-      <c r="C209" t="inlineStr"/>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U891           </t>
-        </is>
-      </c>
-      <c r="E209" t="inlineStr">
-        <is>
-          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
-        </is>
-      </c>
-      <c r="F209" t="inlineStr"/>
-      <c r="G209" t="inlineStr">
-        <is>
-          <t>03/11/2031</t>
-        </is>
-      </c>
-      <c r="H209" t="inlineStr">
-        <is>
-          <t>1874</t>
-        </is>
-      </c>
-      <c r="I209" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="J209" t="inlineStr">
-        <is>
-          <t>110226132440294</t>
-        </is>
-      </c>
-      <c r="K209" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M209" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="N209" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>CAL-001-001-001</t>
-        </is>
-      </c>
-      <c r="C210" t="inlineStr"/>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U948-1         </t>
-        </is>
-      </c>
-      <c r="E210" t="inlineStr">
-        <is>
-          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
-        </is>
-      </c>
-      <c r="F210" t="inlineStr"/>
-      <c r="G210" t="inlineStr">
-        <is>
-          <t>31/01/2032</t>
-        </is>
-      </c>
-      <c r="H210" t="inlineStr">
-        <is>
-          <t>1963</t>
-        </is>
-      </c>
-      <c r="I210" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="J210" t="inlineStr">
-        <is>
-          <t>100826061846740</t>
-        </is>
-      </c>
-      <c r="K210" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L210" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M210" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="N210" t="inlineStr">
         <is>
           <t>NO</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 16/09/2026 09:49:25
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-026-006-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4417,12 +4417,12 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4481,12 +4481,12 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -6379,12 +6379,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6571,12 +6571,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C97" t="inlineStr"/>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -7499,12 +7499,12 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 16/09/2026 14:22:43
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -784,7 +784,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -976,7 +976,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1803,12 +1803,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916050</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916050</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2187,12 +2187,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2251,12 +2251,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2315,12 +2315,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916222</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916222</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3009,22 +3009,22 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3265,22 +3265,22 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3504,7 +3504,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -4161,12 +4161,12 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,12 +4289,12 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4673,12 +4673,12 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4929,22 +4929,22 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5121,12 +5121,12 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5313,12 +5313,12 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5569,12 +5569,12 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5707,12 +5707,12 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5761,12 +5761,12 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5825,12 +5825,12 @@
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5899,12 +5899,12 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -5931,12 +5931,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6091,12 +6091,12 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6123,12 +6123,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6315,12 +6315,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6379,12 +6379,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6411,12 +6411,12 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6507,12 +6507,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6635,12 +6635,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6731,12 +6731,12 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6800,12 +6800,12 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6913,27 +6913,27 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7041,27 +7041,27 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,27 +7233,27 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7297,27 +7297,27 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7361,27 +7361,27 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7425,27 +7425,27 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7809,27 +7809,27 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -7873,27 +7873,27 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7952,12 +7952,12 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -8001,27 +8001,27 @@
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8129,27 +8129,27 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8193,27 +8193,27 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8321,27 +8321,27 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8385,27 +8385,27 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8513,27 +8513,27 @@
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -8543,7 +8543,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8705,27 +8705,27 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8897,27 +8897,27 @@
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
@@ -8927,7 +8927,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9025,27 +9025,27 @@
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -9055,7 +9055,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9195,12 +9195,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9281,27 +9281,27 @@
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -9451,12 +9451,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9515,12 +9515,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
@@ -9552,7 +9552,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9579,12 +9579,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
@@ -9616,7 +9616,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9729,27 +9729,27 @@
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9857,27 +9857,27 @@
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
@@ -9887,7 +9887,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -9921,27 +9921,27 @@
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -9985,27 +9985,27 @@
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1895</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10251,12 +10251,12 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10384,7 +10384,7 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10443,12 +10443,12 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>200226070819709</t>
+          <t>200226062756258</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10960,7 +10960,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226062756258</t>
+          <t>200226070819709</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11713,22 +11713,22 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11777,22 +11777,22 @@
       <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -12033,22 +12033,22 @@
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12097,22 +12097,22 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1922</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1922</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12363,12 +12363,12 @@
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12427,12 +12427,12 @@
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12491,12 +12491,12 @@
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12747,12 +12747,12 @@
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
@@ -13057,22 +13057,22 @@
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -13087,7 +13087,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
@@ -13104,7 +13104,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
@@ -13121,22 +13121,22 @@
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
@@ -13360,7 +13360,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
@@ -13377,22 +13377,22 @@
       <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1860</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
@@ -13407,7 +13407,7 @@
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N203" t="inlineStr">
@@ -13424,7 +13424,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
@@ -13441,22 +13441,22 @@
       <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K204" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
@@ -13552,7 +13552,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C206" t="inlineStr"/>
@@ -13569,27 +13569,27 @@
       <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
-          <t>09/12/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1874</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>180626072347907</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L206" t="inlineStr">
@@ -13599,7 +13599,7 @@
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N206" t="inlineStr">
@@ -13616,7 +13616,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C207" t="inlineStr"/>
@@ -13633,27 +13633,27 @@
       <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>09/12/2031</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>180626072347907</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L207" t="inlineStr">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="N207" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 17/09/2026 06:00:52
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1813</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1949</t>
+          <t>1948</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1949</t>
+          <t>1948</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1949</t>
+          <t>1948</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>1998</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1846</t>
+          <t>1845</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1917</t>
+          <t>1916</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1917</t>
+          <t>1916</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1776</t>
+          <t>1775</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1776</t>
+          <t>1775</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1895</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1844</t>
+          <t>1843</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1922</t>
+          <t>1921</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1964</t>
+          <t>1963</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1922</t>
+          <t>1921</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>1949</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1791</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1860</t>
+          <t>1859</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1874</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>1963</t>
+          <t>1962</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 17/09/2026 15:45:59
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,22 +513,22 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1937</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1937</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,12 +769,12 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -843,12 +843,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -907,12 +907,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1937</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1803,12 +1803,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2753,22 +2753,22 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2945,22 +2945,22 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3137,22 +3137,22 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3777,27 +3777,27 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3841,27 +3841,27 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4225,12 +4225,12 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,12 +4289,12 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4673,12 +4673,12 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4801,12 +4801,12 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4875,12 +4875,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4929,12 +4929,12 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5121,12 +5121,12 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5249,12 +5249,12 @@
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5377,12 +5377,12 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5505,12 +5505,12 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5633,12 +5633,12 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1873</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5707,12 +5707,12 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5835,12 +5835,12 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -6027,12 +6027,12 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6315,12 +6315,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6379,12 +6379,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6657,27 +6657,27 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6721,27 +6721,27 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,12 +7248,12 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7297,27 +7297,27 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7617,27 +7617,27 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7681,27 +7681,27 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -7760,12 +7760,12 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8129,27 +8129,27 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8385,27 +8385,27 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8641,27 +8641,27 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9153,27 +9153,27 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9345,27 +9345,27 @@
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -9375,7 +9375,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
@@ -9409,27 +9409,27 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9456,7 +9456,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
@@ -9473,27 +9473,27 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -9537,27 +9537,27 @@
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -9567,7 +9567,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -9601,27 +9601,27 @@
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9729,27 +9729,27 @@
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1894</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -10059,12 +10059,12 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10187,12 +10187,12 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/09/2026 05:55:19
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,22 +513,22 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1937</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -710,17 +710,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1937</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,12 +769,12 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -838,17 +838,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -902,17 +902,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1937</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1937</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1811</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1776</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1948</t>
+          <t>1947</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1734,17 +1734,17 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1948</t>
+          <t>1947</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1798,17 +1798,17 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1948</t>
+          <t>1947</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2118,17 +2118,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2374,17 +2374,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1845</t>
+          <t>1844</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2753,22 +2753,22 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2945,22 +2945,22 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3137,22 +3137,22 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1857</t>
+          <t>1856</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1916</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1916</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1775</t>
+          <t>1774</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1775</t>
+          <t>1774</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3777,27 +3777,27 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3841,27 +3841,27 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1776</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4225,12 +4225,12 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,12 +4289,12 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4673,12 +4673,12 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4801,12 +4801,12 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4870,17 +4870,17 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4929,12 +4929,12 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5121,12 +5121,12 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5249,12 +5249,12 @@
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5377,12 +5377,12 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5505,12 +5505,12 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5633,12 +5633,12 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5702,17 +5702,17 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5830,17 +5830,17 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,17 +6022,17 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6315,12 +6315,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6379,12 +6379,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6657,27 +6657,27 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6721,27 +6721,27 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7248,12 +7248,12 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7297,27 +7297,27 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7558,17 +7558,17 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7617,27 +7617,27 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7681,27 +7681,27 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7760,12 +7760,12 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8129,27 +8129,27 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8385,27 +8385,27 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8641,27 +8641,27 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8705,27 +8705,27 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9153,27 +9153,27 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9345,27 +9345,27 @@
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -9375,7 +9375,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
@@ -9409,27 +9409,27 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9456,7 +9456,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
@@ -9473,27 +9473,27 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -9537,27 +9537,27 @@
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -9567,7 +9567,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -9601,27 +9601,27 @@
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9729,27 +9729,27 @@
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1894</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1843</t>
+          <t>1842</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,17 +10054,17 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10182,17 +10182,17 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1921</t>
+          <t>1920</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1963</t>
+          <t>1962</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1921</t>
+          <t>1920</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1949</t>
+          <t>1948</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1791</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1859</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1857</t>
+          <t>1856</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1892</t>
+          <t>1891</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -13446,7 +13446,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1909</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>1873</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>1962</t>
+          <t>1961</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/09/2026 06:08:31
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,22 +513,22 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,12 +769,12 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -843,12 +843,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -907,12 +907,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1936</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1803,12 +1803,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-001-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104915753</t>
+          <t>170626104916003</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104915800</t>
+          <t>170626104916081</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104915753</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-028-001-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>170626104916003</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>170626104916081</t>
+          <t>170626104915800</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2379,12 +2379,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2753,22 +2753,22 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2945,22 +2945,22 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -3137,22 +3137,22 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3167,7 +3167,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -3201,22 +3201,22 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3777,27 +3777,27 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1871</t>
+          <t>1776</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3841,27 +3841,27 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1776</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4225,12 +4225,12 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,12 +4289,12 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4673,12 +4673,12 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4801,12 +4801,12 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4875,12 +4875,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5121,12 +5121,12 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5377,12 +5377,12 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5505,12 +5505,12 @@
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5633,12 +5633,12 @@
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5707,12 +5707,12 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5835,12 +5835,12 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -6027,12 +6027,12 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6315,12 +6315,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6379,12 +6379,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6657,27 +6657,27 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -6849,27 +6849,27 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,12 +7248,12 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7297,27 +7297,27 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7563,12 +7563,12 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7617,27 +7617,27 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7681,27 +7681,27 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -7760,12 +7760,12 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8129,27 +8129,27 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8385,27 +8385,27 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8641,27 +8641,27 @@
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8705,27 +8705,27 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -9153,27 +9153,27 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9345,27 +9345,27 @@
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -9375,7 +9375,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
@@ -9409,27 +9409,27 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -9456,7 +9456,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
@@ -9473,27 +9473,27 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -9537,27 +9537,27 @@
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -9567,7 +9567,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -9601,27 +9601,27 @@
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9729,27 +9729,27 @@
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9936,7 +9936,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -10059,12 +10059,12 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>130226105905407</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -10187,12 +10187,12 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905407</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/09/2026 07:01:20
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -11073,22 +11073,22 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/09/2026 07:40:51
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N202"/>
+  <dimension ref="A1:N201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,12 +513,12 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -619,12 +619,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,12 +641,12 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-027-004-003</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1995,12 +1995,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>170626104915925</t>
+          <t>170626104915784</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>170626104916237</t>
+          <t>170626104915925</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-027-004-003</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>170626104915784</t>
+          <t>170626104916237</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2305,22 +2305,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>110226132440591</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2561,22 +2561,22 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439919</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2753,22 +2753,22 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -2881,22 +2881,22 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440591</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2945,22 +2945,22 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>110226132439919</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -3073,22 +3073,22 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3521,27 +3521,27 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1871</t>
+          <t>1776</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3585,27 +3585,27 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1776</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -3615,7 +3615,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3713,12 +3713,12 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3905,12 +3905,12 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4161,12 +4161,12 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4225,12 +4225,12 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,22 +4289,22 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4417,12 +4417,12 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4491,12 +4491,12 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4511,7 +4511,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4865,22 +4865,22 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,12 +5057,12 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5121,12 +5121,12 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5195,12 +5195,12 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5249,12 +5249,12 @@
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5313,12 +5313,12 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5675,12 +5675,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C83" t="inlineStr"/>
@@ -5707,12 +5707,12 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -5899,12 +5899,12 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -5931,12 +5931,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6059,12 +6059,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C89" t="inlineStr"/>
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6187,12 +6187,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6337,22 +6337,22 @@
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6465,27 +6465,27 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6603,12 +6603,12 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6657,27 +6657,27 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,27 +6785,27 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -6849,27 +6849,27 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6992,12 +6992,12 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,27 +7233,27 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,27 +7361,27 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7553,27 +7553,27 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7681,27 +7681,27 @@
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1893</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -7711,7 +7711,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -11073,22 +11073,22 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11696,39 +11696,39 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO101P-1      </t>
+          <t xml:space="preserve">INO102-1       </t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA ACQUA PLUS                             </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>01/02/2032</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1962</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>110826062045431</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11787,12 +11787,12 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11851,12 +11851,12 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11915,12 +11915,12 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1920</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12022,33 +12022,33 @@
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-1       </t>
+          <t xml:space="preserve">INO102-2       </t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA LOFT                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
         </is>
       </c>
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1920</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -12107,12 +12107,12 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12144,39 +12144,39 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO102-2       </t>
+          <t xml:space="preserve">INO103-2       </t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA LOFT                            </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>MMQT4</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12208,39 +12208,39 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO103-2       </t>
+          <t xml:space="preserve">INO104-1       </t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA URBAN                           </t>
+          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
         </is>
       </c>
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>MMQT4</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12363,12 +12363,12 @@
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12406,12 +12406,12 @@
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-1       </t>
+          <t xml:space="preserve">INO104-2       </t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLANCO C/ASIENTO LINEA STONE                                  </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
         </is>
       </c>
       <c r="F188" t="inlineStr"/>
@@ -12427,12 +12427,12 @@
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056680</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>19</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12528,39 +12528,39 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104-2       </t>
+          <t xml:space="preserve">INO104N-1      </t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLANCO LINEA STONE                           </t>
+          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
         </is>
       </c>
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1948</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>180226073056680</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1948</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12656,7 +12656,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
@@ -12673,22 +12673,22 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
@@ -12720,7 +12720,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
@@ -12737,22 +12737,22 @@
       <c r="F193" t="inlineStr"/>
       <c r="G193" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -12767,7 +12767,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N193" t="inlineStr">
@@ -12784,7 +12784,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
@@ -12801,22 +12801,22 @@
       <c r="F194" t="inlineStr"/>
       <c r="G194" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
@@ -12848,39 +12848,39 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-1      </t>
+          <t xml:space="preserve">INO104N-2      </t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t xml:space="preserve">INODORO BLACK C/ASIENTO LINEA STONE                                   </t>
+          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
         </is>
       </c>
       <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1856</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N195" t="inlineStr">
@@ -12912,7 +12912,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
@@ -12929,22 +12929,22 @@
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
@@ -12976,39 +12976,39 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr">
         <is>
-          <t xml:space="preserve">INO104N-2      </t>
+          <t xml:space="preserve">U1133G         </t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t xml:space="preserve">DEPOSITO C/DESCARGA DUAL BLACK LINEA STONE                            </t>
+          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
       <c r="G197" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>22/11/2031</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1891</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>300</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -13023,7 +13023,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>300</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
@@ -13046,28 +13046,28 @@
       <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr">
         <is>
-          <t xml:space="preserve">U1133G         </t>
+          <t xml:space="preserve">U889-01        </t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>U1133G - CAMPANA CUADRADA SOPORTE DUCHADOR MONOC GOLD FABRIC</t>
+          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
         </is>
       </c>
       <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
-          <t>22/11/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>77</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -13087,7 +13087,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>77</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
@@ -13104,7 +13104,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
@@ -13121,27 +13121,27 @@
       <c r="F199" t="inlineStr"/>
       <c r="G199" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>09/12/2031</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1908</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>180626072347907</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>50</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -13168,44 +13168,44 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-027-008-001</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
-          <t xml:space="preserve">U889-01        </t>
+          <t xml:space="preserve">U891           </t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>U889-01 - CAMPANA SANTANDER STD. IMPORTADA</t>
+          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
         </is>
       </c>
       <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
-          <t>09/12/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>180626072347907</t>
+          <t>110226132440294</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L200" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
@@ -13232,39 +13232,39 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>CAL-027-008-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr">
         <is>
-          <t xml:space="preserve">U891           </t>
+          <t xml:space="preserve">U948-1         </t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>U891 - CAMPANA CUADRADA CAÑO FLOR DE DUCHA SANTANDER</t>
+          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
         </is>
       </c>
       <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>31/01/2032</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1961</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>507</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>110226132440294</t>
+          <t>100826061846740</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -13279,74 +13279,10 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>507</t>
         </is>
       </c>
       <c r="N201" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>CALIDAD</t>
-        </is>
-      </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>CAL-001-001-001</t>
-        </is>
-      </c>
-      <c r="C202" t="inlineStr"/>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t xml:space="preserve">U948-1         </t>
-        </is>
-      </c>
-      <c r="E202" t="inlineStr">
-        <is>
-          <t>U948-1 - CAÑO BAJADA DUCHA DE EMB PLASTICO ER 1/2" SR 1/2" 3/4"</t>
-        </is>
-      </c>
-      <c r="F202" t="inlineStr"/>
-      <c r="G202" t="inlineStr">
-        <is>
-          <t>31/01/2032</t>
-        </is>
-      </c>
-      <c r="H202" t="inlineStr">
-        <is>
-          <t>1961</t>
-        </is>
-      </c>
-      <c r="I202" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="J202" t="inlineStr">
-        <is>
-          <t>100826061846740</t>
-        </is>
-      </c>
-      <c r="K202" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="L202" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M202" t="inlineStr">
-        <is>
-          <t>507</t>
-        </is>
-      </c>
-      <c r="N202" t="inlineStr">
         <is>
           <t>NO</t>
         </is>

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 18/09/2026 10:19:19
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -4801,12 +4801,12 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1872</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4865,12 +4865,12 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -5547,12 +5547,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5611,12 +5611,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -11073,22 +11073,22 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1858</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1790</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1788</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 19/09/2026 05:28:13
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>1935</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>1935</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>1935</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1936</t>
+          <t>1935</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1871</t>
+          <t>1870</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1811</t>
+          <t>1810</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1776</t>
+          <t>1775</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1947</t>
+          <t>1946</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1947</t>
+          <t>1946</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1947</t>
+          <t>1946</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1996</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1907</t>
+          <t>1906</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1844</t>
+          <t>1843</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1915</t>
+          <t>1914</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1915</t>
+          <t>1914</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1774</t>
+          <t>1773</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1774</t>
+          <t>1773</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1776</t>
+          <t>1775</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1871</t>
+          <t>1870</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1893</t>
+          <t>1892</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1836</t>
+          <t>1835</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1841</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1920</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1980</t>
+          <t>1979</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1857</t>
+          <t>1856</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1920</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1948</t>
+          <t>1947</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1790</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1858</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>1908</t>
+          <t>1907</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>1872</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>1961</t>
+          <t>1960</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 19/09/2026 07:24:12
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -4801,12 +4801,12 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1871</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4865,12 +4865,12 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1871</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -5547,12 +5547,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5611,12 +5611,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -11073,22 +11073,22 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1857</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1857</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 19/09/2026 09:23:12
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -10928,7 +10928,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1857</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -11073,22 +11073,22 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11248,7 +11248,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1857</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1857</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1789</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1789</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 21/09/2026 05:53:23
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1934</t>
+          <t>1933</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1934</t>
+          <t>1933</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1934</t>
+          <t>1933</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1934</t>
+          <t>1933</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1809</t>
+          <t>1808</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1774</t>
+          <t>1773</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1944</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1944</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1944</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1905</t>
+          <t>1904</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1842</t>
+          <t>1841</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1912</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1913</t>
+          <t>1912</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1772</t>
+          <t>1771</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1772</t>
+          <t>1771</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1774</t>
+          <t>1773</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1891</t>
+          <t>1890</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1834</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1918</t>
+          <t>1917</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1886</t>
+          <t>1885</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1886</t>
+          <t>1885</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1977</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1781</t>
+          <t>1780</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1918</t>
+          <t>1917</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1946</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1788</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1906</t>
+          <t>1905</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1870</t>
+          <t>1869</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1959</t>
+          <t>1958</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 21/09/2026 06:33:57
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -10443,12 +10443,12 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10507,12 +10507,12 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10527,7 +10527,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
@@ -10753,22 +10753,22 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10817,22 +10817,22 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
@@ -10881,22 +10881,22 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -11073,22 +11073,22 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11275,12 +11275,12 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11393,22 +11393,22 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12400,7 +12400,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12464,7 +12464,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 21/09/2026 08:55:29
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -10443,12 +10443,12 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10507,12 +10507,12 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10527,7 +10527,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
@@ -10753,22 +10753,22 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10817,22 +10817,22 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
@@ -10881,22 +10881,22 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
@@ -11073,22 +11073,22 @@
       <c r="F167" t="inlineStr"/>
       <c r="G167" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N167" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11275,12 +11275,12 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11393,22 +11393,22 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12336,7 +12336,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12400,7 +12400,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12464,7 +12464,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 22/09/2026 06:00:45
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1933</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1933</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1933</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1933</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1808</t>
+          <t>1807</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1773</t>
+          <t>1772</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1994</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1904</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1841</t>
+          <t>1840</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1912</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1912</t>
+          <t>1911</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1771</t>
+          <t>1770</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1771</t>
+          <t>1770</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1773</t>
+          <t>1772</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1890</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1917</t>
+          <t>1916</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1885</t>
+          <t>1884</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1885</t>
+          <t>1884</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1977</t>
+          <t>1976</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1780</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1917</t>
+          <t>1916</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>1944</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1905</t>
+          <t>1904</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1869</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12998,7 +12998,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>1958</t>
+          <t>1957</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 22/09/2026 14:36:42
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -592,7 +592,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -641,22 +641,22 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-003-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726111523883</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-027-003-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1803,12 +1803,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>270726111523883</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2177,22 +2177,22 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2241,22 +2241,22 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2305,22 +2305,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2369,22 +2369,22 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2433,22 +2433,22 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2561,22 +2561,22 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2689,22 +2689,22 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -2817,22 +2817,22 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3467,12 +3467,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3585,12 +3585,12 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3777,12 +3777,12 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4033,12 +4033,12 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4097,22 +4097,22 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,12 +4289,12 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4417,12 +4417,12 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4481,12 +4481,12 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4545,12 +4545,12 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4673,12 +4673,12 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4875,12 +4875,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,22 +4993,22 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5185,12 +5185,12 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5291,12 +5291,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5483,12 +5483,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5643,12 +5643,12 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5771,12 +5771,12 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -6017,27 +6017,27 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6081,27 +6081,27 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -6337,27 +6337,27 @@
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -6367,7 +6367,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -6411,12 +6411,12 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,12 +6544,12 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -6593,27 +6593,27 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,27 +6785,27 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -6849,22 +6849,22 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6913,27 +6913,27 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7169,27 +7169,27 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7297,27 +7297,27 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7361,27 +7361,27 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7617,27 +7617,27 @@
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7937,27 +7937,27 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8321,27 +8321,27 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8513,27 +8513,27 @@
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -8543,7 +8543,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8747,12 +8747,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8833,27 +8833,27 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -8875,12 +8875,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C133" t="inlineStr"/>
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9217,27 +9217,27 @@
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -9247,7 +9247,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9675,12 +9675,12 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -9739,12 +9739,12 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10443,12 +10443,12 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10507,12 +10507,12 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10527,7 +10527,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
@@ -10753,22 +10753,22 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10817,22 +10817,22 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10955,12 +10955,12 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11019,12 +11019,12 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11275,12 +11275,12 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11531,12 +11531,12 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11585,22 +11585,22 @@
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1916</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11659,12 +11659,12 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11713,22 +11713,22 @@
       <c r="F177" t="inlineStr"/>
       <c r="G177" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1916</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11787,12 +11787,12 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
@@ -11851,12 +11851,12 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12033,22 +12033,22 @@
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12107,12 +12107,12 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -12368,7 +12368,7 @@
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12560,7 +12560,7 @@
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
@@ -12656,7 +12656,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
@@ -12673,22 +12673,22 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -12703,7 +12703,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 22/09/2026 15:16:33
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,12 +833,12 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1932</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2113,22 +2113,22 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2241,22 +2241,22 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2305,22 +2305,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2497,22 +2497,22 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3201,27 +3201,27 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1772</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3265,27 +3265,27 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1772</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3393,12 +3393,12 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3777,12 +3777,12 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3905,12 +3905,12 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4097,12 +4097,12 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4225,12 +4225,12 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4353,22 +4353,22 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4811,12 +4811,12 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4865,12 +4865,12 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4929,12 +4929,12 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1868</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,12 +5057,12 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5121,12 +5121,12 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1779</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5163,12 +5163,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5227,12 +5227,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5291,12 +5291,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5355,12 +5355,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5515,12 +5515,12 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5547,12 +5547,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -5579,12 +5579,12 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5611,12 +5611,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5739,12 +5739,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5867,12 +5867,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5963,12 +5963,12 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6017,22 +6017,22 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,27 +6209,27 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6273,27 +6273,27 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,27 +6401,27 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,27 +6593,27 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6657,27 +6657,27 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6721,27 +6721,27 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6800,12 +6800,12 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6849,27 +6849,27 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6913,27 +6913,27 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -7041,27 +7041,27 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,27 +7233,27 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7297,27 +7297,27 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7553,27 +7553,27 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7873,27 +7873,27 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8193,27 +8193,27 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8449,27 +8449,27 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8683,12 +8683,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
@@ -8705,27 +8705,27 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8752,7 +8752,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1889</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -9153,27 +9153,27 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1832</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9611,12 +9611,12 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9675,12 +9675,12 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -10315,12 +10315,12 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10443,12 +10443,12 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
@@ -10625,22 +10625,22 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10753,22 +10753,22 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10891,12 +10891,12 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10955,12 +10955,12 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11403,12 +11403,12 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1916</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11595,12 +11595,12 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1916</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11723,12 +11723,12 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11787,12 +11787,12 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12304,7 +12304,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1786</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12496,7 +12496,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1854</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 23/09/2026 06:08:30
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -646,17 +646,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -838,17 +838,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1932</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1807</t>
+          <t>1806</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,17 +1350,17 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,17 +1478,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1772</t>
+          <t>1771</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1670,17 +1670,17 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1734,17 +1734,17 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>1992</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1840</t>
+          <t>1839</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2305,22 +2305,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2753,22 +2753,22 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1911</t>
+          <t>1910</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1770</t>
+          <t>1769</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1770</t>
+          <t>1769</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1772</t>
+          <t>1771</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3457,12 +3457,12 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3969,12 +3969,12 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4097,12 +4097,12 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,12 +4289,12 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4358,17 +4358,17 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4545,12 +4545,12 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4678,17 +4678,17 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,12 +5057,12 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1889</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1832</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1838</t>
+          <t>1837</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1916</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1884</t>
+          <t>1883</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1884</t>
+          <t>1883</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1976</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,17 +10374,17 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10438,17 +10438,17 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10800,7 +10800,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
@@ -10817,22 +10817,22 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
@@ -10881,22 +10881,22 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,17 +11142,17 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11206,17 +11206,17 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11393,22 +11393,22 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11462,17 +11462,17 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1916</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11718,17 +11718,17 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11782,17 +11782,17 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12038,17 +12038,17 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1786</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12400,7 +12400,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12464,7 +12464,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1854</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1886</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1904</t>
+          <t>1903</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1868</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1957</t>
+          <t>1956</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 23/09/2026 06:35:00
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -523,12 +523,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -651,12 +651,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -843,12 +843,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2305,22 +2305,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2753,22 +2753,22 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3457,12 +3457,12 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3969,12 +3969,12 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4033,22 +4033,22 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4097,12 +4097,12 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4289,12 +4289,12 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4363,12 +4363,12 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4545,12 +4545,12 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4683,12 +4683,12 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,12 +5057,12 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10443,12 +10443,12 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226062905996</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10576,7 +10576,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226062905996</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>280426082846940</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10800,7 +10800,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
@@ -10817,22 +10817,22 @@
       <c r="F163" t="inlineStr"/>
       <c r="G163" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>280426082846940</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
@@ -10881,22 +10881,22 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10992,7 +10992,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
@@ -11009,22 +11009,22 @@
       <c r="F166" t="inlineStr"/>
       <c r="G166" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11265,22 +11265,22 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N170" t="inlineStr">
@@ -11329,22 +11329,22 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11393,22 +11393,22 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1915</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11600,7 +11600,7 @@
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11723,12 +11723,12 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11787,12 +11787,12 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-003-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/01/2032</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>280726145222369</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -12272,7 +12272,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
@@ -12289,22 +12289,22 @@
       <c r="F186" t="inlineStr"/>
       <c r="G186" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -12400,7 +12400,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12464,7 +12464,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>CAL-003-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
@@ -12481,22 +12481,22 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>18/01/2032</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>280726145222369</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 23/09/2026 11:14:54
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,12 +833,12 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2113,22 +2113,22 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2241,22 +2241,22 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2305,22 +2305,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2497,22 +2497,22 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3201,27 +3201,27 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1771</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3265,27 +3265,27 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1771</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3393,12 +3393,12 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3777,12 +3777,12 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3905,12 +3905,12 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4097,12 +4097,12 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4225,12 +4225,12 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4353,22 +4353,22 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4811,12 +4811,12 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4865,12 +4865,12 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4929,12 +4929,12 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,12 +5057,12 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5121,12 +5121,12 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5163,12 +5163,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5227,12 +5227,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5291,12 +5291,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5355,12 +5355,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5515,12 +5515,12 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5547,12 +5547,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -5579,12 +5579,12 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5611,12 +5611,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5739,12 +5739,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5867,12 +5867,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5963,12 +5963,12 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6017,22 +6017,22 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,27 +6209,27 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6273,27 +6273,27 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,27 +6401,27 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,27 +6593,27 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6657,27 +6657,27 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6721,27 +6721,27 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6800,12 +6800,12 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6849,27 +6849,27 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6913,27 +6913,27 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,27 +7233,27 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7297,27 +7297,27 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7553,27 +7553,27 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7873,27 +7873,27 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8193,27 +8193,27 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8449,27 +8449,27 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8683,12 +8683,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
@@ -8705,27 +8705,27 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8752,7 +8752,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -9153,27 +9153,27 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9611,12 +9611,12 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9675,12 +9675,12 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -10315,12 +10315,12 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10443,12 +10443,12 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
@@ -10625,22 +10625,22 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10753,22 +10753,22 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10891,12 +10891,12 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10955,12 +10955,12 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11403,12 +11403,12 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11595,12 +11595,12 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1915</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11723,12 +11723,12 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11787,12 +11787,12 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12304,7 +12304,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12496,7 +12496,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1851</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 23/09/2026 11:28:11
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAL-027-006-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>160726135002875</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAL-027-005-003</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>160726135002890</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,12 +833,12 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -875,12 +875,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -939,12 +939,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-005-003</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -961,22 +961,22 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002890</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-006-003</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1025,22 +1025,22 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002875</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440341</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1483,12 +1483,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>110226132440341</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAL-027-002-003</t>
+          <t>CAL-027-001-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1675,12 +1675,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>270726063454949</t>
+          <t>270726111523899</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>180</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CAL-027-001-003</t>
+          <t>CAL-027-002-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1739,12 +1739,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>270726111523899</t>
+          <t>270726063454949</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>140</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-027-003-001</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2113,22 +2113,22 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519010</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2241,22 +2241,22 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2305,22 +2305,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CAL-027-007-001</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -2497,22 +2497,22 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>130526104518979</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CAL-027-003-001</t>
+          <t>CAL-027-007-001</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -2768,7 +2768,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>130526104519010</t>
+          <t>130526104518979</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3201,27 +3201,27 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>02/11/2031</t>
+          <t>30/07/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1771</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110526091026715</t>
+          <t>060226072431854</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3265,27 +3265,27 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>30/07/2031</t>
+          <t>02/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1771</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>060226072431854</t>
+          <t>110526091026715</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3393,12 +3393,12 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3713,22 +3713,22 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3743,7 +3743,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3777,12 +3777,12 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3841,22 +3841,22 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3905,12 +3905,12 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4097,12 +4097,12 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4225,12 +4225,12 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4353,22 +4353,22 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4609,12 +4609,12 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4811,12 +4811,12 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4865,12 +4865,12 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4929,12 +4929,12 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -4993,12 +4993,12 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1867</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5057,12 +5057,12 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5121,12 +5121,12 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1778</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5163,12 +5163,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -5227,12 +5227,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CAL-028-007-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>030626072815492</t>
+          <t>030626072815555</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5291,12 +5291,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-007-002</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815492</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5355,12 +5355,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>030626072815555</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5515,12 +5515,12 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5547,12 +5547,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -5579,12 +5579,12 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5611,12 +5611,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C82" t="inlineStr"/>
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -5739,12 +5739,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -5776,7 +5776,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5867,12 +5867,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5963,12 +5963,12 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6017,22 +6017,22 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6047,7 +6047,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -6209,27 +6209,27 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6273,27 +6273,27 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -6303,7 +6303,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -6401,27 +6401,27 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>070426090312179</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,27 +6593,27 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6657,27 +6657,27 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6721,27 +6721,27 @@
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6800,12 +6800,12 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6849,27 +6849,27 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6913,27 +6913,27 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>070426090312179</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7056,7 +7056,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7233,27 +7233,27 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -7297,27 +7297,27 @@
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -7327,7 +7327,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7553,27 +7553,27 @@
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7873,27 +7873,27 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8193,27 +8193,27 @@
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8449,27 +8449,27 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>070426090312413</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8656,7 +8656,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8683,12 +8683,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
@@ -8705,27 +8705,27 @@
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -8735,7 +8735,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8752,7 +8752,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1888</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8811,12 +8811,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>070426090312413</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -9153,27 +9153,27 @@
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1831</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9232,7 +9232,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9611,12 +9611,12 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905391</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9675,12 +9675,12 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>130226105905391</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -10315,12 +10315,12 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -10443,12 +10443,12 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
@@ -10625,22 +10625,22 @@
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -10672,7 +10672,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
@@ -10689,22 +10689,22 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>200226062756274</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -10753,22 +10753,22 @@
       <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>200226062756274</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10891,12 +10891,12 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10955,12 +10955,12 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11147,12 +11147,12 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11211,12 +11211,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11403,12 +11403,12 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11467,12 +11467,12 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1915</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11595,12 +11595,12 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -11615,7 +11615,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -11723,12 +11723,12 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
@@ -11787,12 +11787,12 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12043,12 +12043,12 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12304,7 +12304,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>290426062413220</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -12353,22 +12353,22 @@
       <c r="F187" t="inlineStr"/>
       <c r="G187" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1785</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -12417,22 +12417,22 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1783</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -12496,7 +12496,7 @@
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>290426062413220</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -12528,7 +12528,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
@@ -12545,22 +12545,22 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N190" t="inlineStr">
@@ -12592,7 +12592,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
@@ -12609,22 +12609,22 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1851</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -12639,7 +12639,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 24/09/2026 02:56:29
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1865</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1806</t>
+          <t>1805</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1771</t>
+          <t>1770</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>1991</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1902</t>
+          <t>1901</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1839</t>
+          <t>1838</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1851</t>
+          <t>1850</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1910</t>
+          <t>1909</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1769</t>
+          <t>1768</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1769</t>
+          <t>1768</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1771</t>
+          <t>1770</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1865</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3654,7 +3654,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4230,7 +4230,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5062,7 +5062,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6790,7 +6790,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7366,7 +7366,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7430,7 +7430,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7494,7 +7494,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8198,7 +8198,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8326,7 +8326,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8390,7 +8390,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8454,7 +8454,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8518,7 +8518,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8582,7 +8582,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8838,7 +8838,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>1888</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>1831</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>1837</t>
+          <t>1836</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9478,7 +9478,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9542,7 +9542,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9798,7 +9798,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>1915</t>
+          <t>1914</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9990,7 +9990,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>1883</t>
+          <t>1882</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>1883</t>
+          <t>1882</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -10118,7 +10118,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>1974</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -10374,7 +10374,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10438,7 +10438,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10694,7 +10694,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10822,7 +10822,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10886,7 +10886,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10950,7 +10950,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -11078,7 +11078,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>1778</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11654,7 +11654,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1915</t>
+          <t>1914</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11718,7 +11718,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -11974,7 +11974,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -12358,7 +12358,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>1785</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>1783</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>1851</t>
+          <t>1850</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>1886</t>
+          <t>1885</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>1903</t>
+          <t>1902</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>1867</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>1956</t>
+          <t>1955</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 24/09/2026 08:27:17
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,22 +513,22 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1227,12 +1227,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1793,22 +1793,22 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1985,22 +1985,22 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2049,22 +2049,22 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2113,22 +2113,22 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2177,22 +2177,22 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2241,22 +2241,22 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2305,22 +2305,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2369,22 +2369,22 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3201,12 +3201,12 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,12 +3265,12 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3329,12 +3329,12 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3457,12 +3457,12 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3649,12 +3649,12 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3713,12 +3713,12 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3915,12 +3915,12 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3969,12 +3969,12 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4353,12 +4353,12 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4673,12 +4673,12 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4843,12 +4843,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -4875,12 +4875,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -5067,12 +5067,12 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5099,12 +5099,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5419,12 +5419,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5569,27 +5569,27 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5697,27 +5697,27 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5761,27 +5761,27 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5835,12 +5835,12 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5953,27 +5953,27 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,27 +6081,27 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6145,27 +6145,27 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6209,27 +6209,27 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6288,12 +6288,12 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -6352,12 +6352,12 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -6465,27 +6465,27 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,27 +6593,27 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6657,27 +6657,27 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,27 +6785,27 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -6849,27 +6849,27 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7041,27 +7041,27 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,27 +7361,27 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7425,27 +7425,27 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7809,27 +7809,27 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -7873,27 +7873,27 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7937,27 +7937,27 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8001,27 +8001,27 @@
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -8043,12 +8043,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -8065,27 +8065,27 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8321,27 +8321,27 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8363,12 +8363,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8449,27 +8449,27 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8577,27 +8577,27 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8833,27 +8833,27 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9163,12 +9163,12 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9291,12 +9291,12 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -9931,12 +9931,12 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -10059,12 +10059,12 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10224,7 +10224,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
@@ -10241,22 +10241,22 @@
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10416,7 +10416,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
@@ -10433,22 +10433,22 @@
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10480,7 +10480,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
@@ -10497,22 +10497,22 @@
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10527,7 +10527,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
@@ -10561,22 +10561,22 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -10763,12 +10763,12 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10827,12 +10827,12 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10881,22 +10881,22 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1851</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11019,12 +11019,12 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>200226070820084</t>
+          <t>200226070819912</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11137,22 +11137,22 @@
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>21/12/2031</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1914</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11201,22 +11201,22 @@
       <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>1914</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K169" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -11312,7 +11312,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-027-004-001</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
@@ -11339,12 +11339,12 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>180226073056696</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -11359,7 +11359,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>42</t>
         </is>
       </c>
       <c r="N171" t="inlineStr">
@@ -11376,7 +11376,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>CAL-027-004-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
@@ -11403,12 +11403,12 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>180226073056696</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -11423,7 +11423,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -11521,22 +11521,22 @@
       <c r="F174" t="inlineStr"/>
       <c r="G174" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226062905981</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -11551,7 +11551,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -11649,22 +11649,22 @@
       <c r="F176" t="inlineStr"/>
       <c r="G176" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>200226062905981</t>
+          <t>180226073056649</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -11679,7 +11679,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -11905,22 +11905,22 @@
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>200226062756243</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
@@ -11969,22 +11969,22 @@
       <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413142</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -11999,7 +11999,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -12016,7 +12016,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
@@ -12033,22 +12033,22 @@
       <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>290426062413142</t>
+          <t>200226062756243</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
@@ -12161,22 +12161,22 @@
       <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
-          <t>18/10/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>1850</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>290426062413048</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12191,7 +12191,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
@@ -12225,22 +12225,22 @@
       <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>18/10/2031</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1850</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>290426062413048</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -12255,7 +12255,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">

</xml_diff>

<commit_message>
Actualización automática WMS - Stock Calidad Laboratorio - 24/09/2026 08:53:42
</commit_message>
<xml_diff>
--- a/Data_WMS/Stock Calidad Laboratorio.xlsx
+++ b/Data_WMS/Stock Calidad Laboratorio.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CAL-027-007-003</t>
+          <t>CAL-026-004-002</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -513,22 +513,22 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>160726135002906</t>
+          <t>180226073056524</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>220</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CAL-026-002-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -577,22 +577,22 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>260326122851488</t>
+          <t>060226143406731</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>324</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>060226143406731</t>
+          <t>060226143406762</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -715,12 +715,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>060226143406762</t>
+          <t>060226143406747</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>72</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAL-026-004-002</t>
+          <t>CAL-027-007-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -769,22 +769,22 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>180226073056524</t>
+          <t>160726135002906</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>220</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -811,12 +811,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-008-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -833,22 +833,22 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>06/01/2032</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>060226143406747</t>
+          <t>160726135002921</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>260</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAL-027-008-003</t>
+          <t>CAL-026-002-002</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -897,22 +897,22 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>06/01/2032</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>160726135002921</t>
+          <t>260326122851488</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>186</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1227,12 +1227,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>110226132440325</t>
+          <t>110226132440310</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>100</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>110226132440310</t>
+          <t>110226132440325</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>75</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CAL-026-001-001</t>
+          <t>CAL-026-007-002</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1793,22 +1793,22 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>110226132440575</t>
+          <t>130526104519057</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CAL-027-005-002</t>
+          <t>CAL-027-004-002</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>130526104519072</t>
+          <t>130526104519041</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CAL-027-004-002</t>
+          <t>CAL-026-001-001</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1985,22 +1985,22 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>130526104519041</t>
+          <t>110226132440575</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CAL-027-006-001</t>
+          <t>CAL-027-005-002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -2049,22 +2049,22 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>110226132440544</t>
+          <t>130526104519072</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CAL-026-007-002</t>
+          <t>CAL-027-005-001</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -2113,22 +2113,22 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>130526104519057</t>
+          <t>110226132439669</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CAL-026-004-001</t>
+          <t>CAL-026-006-002</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -2177,22 +2177,22 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>110226132440560</t>
+          <t>130526104518963</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CAL-026-006-002</t>
+          <t>CAL-027-006-001</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -2241,22 +2241,22 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>130526104518963</t>
+          <t>110226132440544</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CAL-027-005-001</t>
+          <t>CAL-026-008-002</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -2305,22 +2305,22 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>110226132439669</t>
+          <t>130526104519088</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>400</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CAL-026-008-002</t>
+          <t>CAL-026-004-001</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -2369,22 +2369,22 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>130526104519088</t>
+          <t>110226132440560</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>130526104518916</t>
+          <t>130526104518885</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>110226132440075</t>
+          <t>130226105905313</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>130226105905532</t>
+          <t>130226105905438</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -3201,12 +3201,12 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>110226132440153</t>
+          <t>130526104518869</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3265,12 +3265,12 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>110226132440138</t>
+          <t>130526104518947</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3329,12 +3329,12 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>130526104518854</t>
+          <t>130226105905516</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>130226105905469</t>
+          <t>110226132440138</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3457,12 +3457,12 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>130526104518932</t>
+          <t>130226105905500</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>130226105905547</t>
+          <t>110226132440153</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>130226105905344</t>
+          <t>130226105905250</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -3649,12 +3649,12 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>110226132440091</t>
+          <t>130526104518854</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -3713,12 +3713,12 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>130526104518885</t>
+          <t>130226105905547</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>130226105905563</t>
+          <t>130226105905344</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -3856,7 +3856,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>130226105905453</t>
+          <t>110226132440075</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -3915,12 +3915,12 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>130526104518822</t>
+          <t>130526104518916</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3969,12 +3969,12 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>130526104518838</t>
+          <t>110226132440091</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>130226105905250</t>
+          <t>130226105905282</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>130226105905516</t>
+          <t>130226105905485</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -4161,22 +4161,22 @@
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>130526104518869</t>
+          <t>110226132440060</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>360</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>110226132440122</t>
+          <t>130226105905532</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>130526104518901</t>
+          <t>130526104518932</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -4353,12 +4353,12 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>03/11/2031</t>
+          <t>06/08/2031</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1866</t>
+          <t>1777</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>130526104518947</t>
+          <t>130226105905469</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>130226105905500</t>
+          <t>110226132440122</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>130226105905282</t>
+          <t>130226105905563</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -4545,22 +4545,22 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>110226132440060</t>
+          <t>130526104518901</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>360</t>
+          <t>480</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4609,22 +4609,22 @@
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>130226105905438</t>
+          <t>130526104518822</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -4639,7 +4639,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>160</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4673,12 +4673,12 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>06/08/2031</t>
+          <t>03/11/2031</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>1777</t>
+          <t>1866</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>130226105905313</t>
+          <t>130526104518838</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -4752,7 +4752,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>130226105905485</t>
+          <t>130226105905453</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CAL-028-006-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -4816,7 +4816,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>030626072815461</t>
+          <t>030626072815446</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -4843,12 +4843,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -4875,12 +4875,12 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>030626072815508</t>
+          <t>030626072815617</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>030626072815446</t>
+          <t>030626072815633</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-028-004-002</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -5067,12 +5067,12 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>030626072815617</t>
+          <t>030626072815539</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5087,7 +5087,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -5099,12 +5099,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-006-002</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>030626072815633</t>
+          <t>030626072815461</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CAL-028-004-002</t>
+          <t>CAL-028-003-002</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>030626072815539</t>
+          <t>030626072815430</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CAL-028-005-002</t>
+          <t>CAL-028-002-002</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>030626072815602</t>
+          <t>030626072815571</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>030626072815524</t>
+          <t>030626072815508</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -5419,12 +5419,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>CAL-028-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>030626072815430</t>
+          <t>030626072815524</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>CAL-028-002-002</t>
+          <t>CAL-028-005-002</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>030626072815571</t>
+          <t>030626072815602</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -5569,27 +5569,27 @@
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>030626072815867</t>
+          <t>070426090312366</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -5599,7 +5599,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>070426090312304</t>
+          <t>060426081147718</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -5697,27 +5697,27 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>070426090312398</t>
+          <t>030626072815680</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5761,27 +5761,27 @@
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>060426081147812</t>
+          <t>030626072815664</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5835,12 +5835,12 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>060426081147671</t>
+          <t>060426081147843</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5855,7 +5855,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>070426090312320</t>
+          <t>070426090311866</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -5953,27 +5953,27 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>030626072815821</t>
+          <t>070426090312304</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -5983,7 +5983,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>070426090312210</t>
+          <t>070426090312273</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -6081,27 +6081,27 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>060426081147796</t>
+          <t>030626072815696</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6145,27 +6145,27 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>030626072815711</t>
+          <t>070426090312460</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6209,27 +6209,27 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>030626072815836</t>
+          <t>070426090312398</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -6239,7 +6239,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -6288,12 +6288,12 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>070426090312351</t>
+          <t>060426081147687</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -6352,12 +6352,12 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>060426081147687</t>
+          <t>070426090312241</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -6465,27 +6465,27 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>070426090311585</t>
+          <t>030626072815711</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>030626072815696</t>
+          <t>030626072815836</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -6593,27 +6593,27 @@
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>070426090312241</t>
+          <t>030626072815586</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6657,27 +6657,27 @@
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>030626072815852</t>
+          <t>070426090312210</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6736,7 +6736,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>070426090312257</t>
+          <t>060426081147781</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -6785,27 +6785,27 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>070426090311866</t>
+          <t>030626072815758</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -6849,27 +6849,27 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>060426081147843</t>
+          <t>030626072815821</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -6879,7 +6879,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>060426081147718</t>
+          <t>060426081147671</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -6977,27 +6977,27 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>030626072815758</t>
+          <t>070426090312320</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -7007,7 +7007,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7041,27 +7041,27 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>030626072815680</t>
+          <t>060426081147812</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -7071,7 +7071,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7105,27 +7105,27 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>030626072815664</t>
+          <t>070426090311585</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>070426090312195</t>
+          <t>070426090312257</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7248,7 +7248,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>030626072815742</t>
+          <t>030626072815852</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7312,7 +7312,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>070426090312273</t>
+          <t>070426090312351</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7361,27 +7361,27 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>030626072815789</t>
+          <t>060426081147796</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7391,7 +7391,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7425,27 +7425,27 @@
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>070426090312226</t>
+          <t>030626072815867</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>060426081147750</t>
+          <t>070426090312195</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>030626072815649</t>
+          <t>030626072815742</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>070426090312445</t>
+          <t>060426081147750</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>030626072815946</t>
+          <t>030626072815789</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>030626072815914</t>
+          <t>030626072815946</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7809,27 +7809,27 @@
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>060426081147703</t>
+          <t>030626072815914</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -7873,27 +7873,27 @@
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>070426090311835</t>
+          <t>030626072815727</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7937,27 +7937,27 @@
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>030626072815727</t>
+          <t>070426090312226</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -7979,12 +7979,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>CAL-028-008-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -8001,27 +8001,27 @@
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>030626072815899</t>
+          <t>060426081147734</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -8043,12 +8043,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>LABORATORIO</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>CAL-027-003-002</t>
+          <t>LAB-001-001-001</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
@@ -8065,27 +8065,27 @@
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>070426090312382</t>
+          <t>030626072815649</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -8095,7 +8095,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>070426090312460</t>
+          <t>070426090312445</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>070426090312366</t>
+          <t>060426081147703</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -8257,27 +8257,27 @@
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>030626072815805</t>
+          <t>070426090311835</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -8299,12 +8299,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-028-008-002</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
@@ -8321,27 +8321,27 @@
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>070426090312335</t>
+          <t>030626072815899</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -8351,7 +8351,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -8363,12 +8363,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LABORATORIO</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>LAB-001-001-001</t>
+          <t>CAL-027-003-002</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -8400,7 +8400,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>070426090312288</t>
+          <t>070426090312382</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8449,27 +8449,27 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>060426081147734</t>
+          <t>030626072815805</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>070426090312429</t>
+          <t>070426090312335</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8577,27 +8577,27 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>030626072815930</t>
+          <t>070426090312429</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -8607,7 +8607,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>060426081147828</t>
+          <t>070426090312288</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8769,27 +8769,27 @@
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28/09/2031</t>
+          <t>24/11/2031</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>1830</t>
+          <t>1887</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>060426081147781</t>
+          <t>030626072815930</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>CALIDAD</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -8833,27 +8833,27 @@
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
-          <t>24/11/2031</t>
+          <t>28/09/2031</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>1887</t>
+          <t>1830</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>030626072815774</t>
+          <t>060426081147765</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>CALIDAD</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -8863,7 +8863,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>060426081147765</t>
+          <t>060426081147828</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>030626072815586</t>
+          <t>030626072815774</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -9163,12 +9163,12 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>130226105905422</t>
+          <t>130226105905375</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>57</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -9291,12 +9291,12 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>130226105905375</t>
+          <t>130226105905422</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9311,7 +9311,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>47</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -9931,12 +9931,12 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>200226070819818</t>
+          <t>200226070820209</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -10059,12 +10059,12 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>200226070820209</t>
+          <t>200226070819818</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -10224,7 +10224,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
@@ -10241,22 +10241,22 @@
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>11/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>1782</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>180226073056633</t>
+          <t>290426062413110</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10416,7 +10416,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
@@ -10433,22 +10433,22 @@
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>11/08/2031</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1782</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>290426062413110</t>
+          <t>180226073056633</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -10463,7 +10463,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -10480,7 +10480,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>CAL-001-001-001</t>
+          <t>CAL-002-001-001</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
@@ -10497,22 +10497,22 @@
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
-          <t>20/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>1852</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>290426062413017</t>
+          <t>200226070819849</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -10527,7 +10527,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>CAL-002-001-001</t>
+          <t>CAL-001-001-001</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
@@ -10561,22 +10561,22 @@
       <c r="F159" t="inlineStr"/>
       <c r="G159" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>20/10/2031</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1852</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>200226070819849</t>
+          <t>290426062413017</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -10763,12 +10763,12 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>200226062756212</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
@@ -10827,12 +10827,12 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N163" t="inlineStr">
@@ -10881,22 +10881,22 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>13/08/2031</t>
+          <t>19/10/2031</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>1784</t>
+          <t>1851</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>180226073056727</t>
+          <t>110326145242639</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -10911,7 +10911,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -10945,22 +10945,22 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>19/10/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>1851</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>110326145242639</t>
+          <t>180226073056727</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -10975,7 +10975,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -11019,12 +11019,12 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>200226070820240</t>
+          <t>200226062756212</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
@@ -11039,7 +11039,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="J167" t="inlineStr">
         <is>
-          <t>200226070819912</t>
+          <t>200226070820084</t>
         </is>
       </c>
       <c r="K167" t="inlineStr">
@@ -11137,22 +11137,22 @@
       <c r="F168" t="inlineStr"/>
       <c r="G168" t="inlineStr">
         <is>
-          <t>21/12/2031</t>
+          <t>13/08/2031</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>1914</t>
+          <t>1784</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
         <is>
-          <t>180226073056649</t>
+          <t>200226070820240</t>
         </is>
       </c>
       <c r="K168" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N168" t="inlineStr">
@@ -11201,22 +11201,22 @@
       <c r="F169"